<commit_message>
added the Customer column to the sales report table
</commit_message>
<xml_diff>
--- a/client/public/Sorce/balanceZP.xlsx
+++ b/client/public/Sorce/balanceZP.xlsx
@@ -14,12 +14,12 @@
 </file>
 
 <file path=xl/SharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="434">
   <si>
     <t>Формирвоание отчета</t>
   </si>
   <si>
-    <t>Период: на 19.03.2026 20:05:29</t>
+    <t>Период: на 05.04.2026 19:35:14</t>
   </si>
   <si>
     <t>Показатели: Свободный остаток(В ед. хранения);</t>
@@ -83,9 +83,15 @@
     <t>Желе ківі УБ 78г /56шт АКЦІЯ</t>
   </si>
   <si>
+    <t>Желе Лісова ягода УБ 78г /56шт</t>
+  </si>
+  <si>
     <t>Желе полуниця УБ 78г /56шт</t>
   </si>
   <si>
+    <t>Какао-порошок 22% УБ 60г /26шт</t>
+  </si>
+  <si>
     <t>Какао-порошок УБ 80г /48шт</t>
   </si>
   <si>
@@ -98,24 +104,18 @@
     <t>Ванілін УБ 2г /98шт</t>
   </si>
   <si>
-    <t>Ванільний цукор УБ 10г /58шт</t>
-  </si>
-  <si>
-    <t>Ванільний цукор УБ 10г /58шт АКЦІЯ</t>
-  </si>
-  <si>
     <t>Глазур декоративна біла УБ 75г /40шт</t>
   </si>
   <si>
+    <t>Глазур декоративна біла УБ 75г /40шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Глазур для паски біла УБ 75г /40шт АКЦІЯ ВІП</t>
   </si>
   <si>
     <t>Желатин УБ 25г /42шт</t>
   </si>
   <si>
-    <t>Желатин УБ 25г /42шт АКЦІЯ</t>
-  </si>
-  <si>
     <t>Лимонна кислота УБ 100г /48шт</t>
   </si>
   <si>
@@ -128,12 +128,21 @@
     <t>Посипка декоративна №1 УБ 7г /55шт</t>
   </si>
   <si>
+    <t>Посипка декоративна №1 УБ 7г /55шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Посипка декоративна №2 УБ 7г /55шт</t>
   </si>
   <si>
+    <t>Посипка декоративна №2 УБ 7г /55шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Посипка декоративна №3 УБ 7г /55шт</t>
   </si>
   <si>
+    <t>Посипка декоративна №3 УБ 7г /55шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Суміш для приготування Грибного соусу УБ 36г /34шт</t>
   </si>
   <si>
@@ -167,18 +176,24 @@
     <t>Приправа до курки УБ 25г /34шт</t>
   </si>
   <si>
-    <t>Приправа до курки УБ 25г /34шт АКЦІЯ ВІП</t>
+    <t>Приправа до м'яса УБ 25г /34шт</t>
   </si>
   <si>
     <t>Приправа до моркви по-корейськи УБ 20г /48шт</t>
   </si>
   <si>
+    <t>Приправа до моркви по-корейськи УБ 20г /48шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Приправа до плову УБ 25г /36шт</t>
   </si>
   <si>
     <t>Приправа до риби УБ 25г /30шт</t>
   </si>
   <si>
+    <t>Приправа до риби УБ 25г /30шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Приправа до шашлику УБ 25г /34шт</t>
   </si>
   <si>
@@ -200,6 +215,9 @@
     <t>Суміш прянощів «Хмелі-сунелі» по-грузинськи УБ 20г /24шт</t>
   </si>
   <si>
+    <t>Суміш прянощів «Хмелі-сунелі» по-грузинськи УБ 20г /24шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Суміш прянощів Італійські трави УБ 10г /28шт</t>
   </si>
   <si>
@@ -254,9 +272,6 @@
     <t>Перець чорний горошком УБ 20г /32шт АКЦІЯ Цінова</t>
   </si>
   <si>
-    <t>Перець чорний мелений УБ 20г /38шт</t>
-  </si>
-  <si>
     <t>Перець чорний мелений УБ 20г /38шт АКЦІЯ Цінова</t>
   </si>
   <si>
@@ -272,6 +287,9 @@
     <t>Батон ROSHEN "Double peanuts" мол-шок з арахісом та арахісовим кремом ВКФ 39г /180шт /</t>
   </si>
   <si>
+    <t>Батон ROSHEN "Double peanuts" мол-шок з арахісом та арахісовим кремом ВКФ 39г /180шт /АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Батон ROSHEN "Double peanuts" мол-шок з арахісом та арахісовим кремом ВКФ 39г /180шт /АКЦІЯ Цінова</t>
   </si>
   <si>
@@ -284,7 +302,7 @@
     <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /</t>
   </si>
   <si>
-    <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /АКЦІЯ Цінова</t>
+    <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /АКЦІЯ ОПТ</t>
   </si>
   <si>
     <t>Батон ROSHEN з начинкою ВКФ 43г /180шт /АКЦІЯ Цінова накладна</t>
@@ -293,12 +311,18 @@
     <t>Батон ROSHEN мол-шок з карамельною начинкою ВКФ 40г /180шт /</t>
   </si>
   <si>
+    <t>Батон ROSHEN мол-шок з карамельною начинкою ВКФ 40г /180шт /АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Батон ROSHEN мол-шок з карамельною начинкою ВКФ 40г /180шт /АКЦІЯ Цінова</t>
   </si>
   <si>
     <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт /</t>
   </si>
   <si>
+    <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт /АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Батон ROSHEN мол-шок з кокосом та мигдалем ВКФ 38г /180шт /АКЦІЯ Цінова</t>
   </si>
   <si>
@@ -311,12 +335,12 @@
     <t>Батон ROSHEN молочно-шоколадний з арахісовою начинкою ВКФ 38г /180шт UA TP</t>
   </si>
   <si>
-    <t>Батон ROSHEN молочно-шоколадний з арахісовою начинкою ВКФ 38г /180шт UA TP АКЦІЯ ОПТ</t>
-  </si>
-  <si>
     <t>Батон ROSHEN молочно-шоколадний з начинкою крем-брюле ВКФ 43г /180шт /</t>
   </si>
   <si>
+    <t>Батон ROSHEN молочно-шоколадний з начинкою крем-брюле ВКФ 43г /180шт /АКЦІЯ ОПТ</t>
+  </si>
+  <si>
     <t>Батон ROSHEN молочно-шоколадний з начинкою крем-брюле ВКФ 43г /180шт /АКЦІЯ Цінова</t>
   </si>
   <si>
@@ -347,6 +371,9 @@
     <t>Тістечка Too Cool Choco Fest ВКФ 270г /12шт</t>
   </si>
   <si>
+    <t>Тістечка Too Cool Milk Party ВКФ 270г /12шт</t>
+  </si>
+  <si>
     <t>Тістечка Too Cool Strawberry Splash ВКФ 270г /12шт</t>
   </si>
   <si>
@@ -356,9 +383,6 @@
     <t>Konafetto cocoa з начинкою крем-какао ВКФ 140г /15шт</t>
   </si>
   <si>
-    <t>Konafetto з ванільною начинкою ВКФ 140г /15шт</t>
-  </si>
-  <si>
     <t>Konafetto з горіховою начинкою ВКФ 140г /15шт</t>
   </si>
   <si>
@@ -383,21 +407,12 @@
     <t>Wafers Sandwich Crunch ваніль ККФ 142г /15шт /</t>
   </si>
   <si>
-    <t>Wafers Sandwich Crunch ваніль ККФ 142г /15шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Wafers Sandwich Crunch горіх ККФ 142г /15шт /</t>
   </si>
   <si>
-    <t>Wafers Sandwich Crunch горіх ККФ 142г /15шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Wafers Sandwich Crunch какао ККФ 142г /15шт /</t>
   </si>
   <si>
-    <t>Wafers Sandwich Crunch какао ККФ 142г /15шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
     <t>Wafers Sandwich Crunch лимон ККФ 142г /15шт /</t>
   </si>
   <si>
@@ -413,36 +428,45 @@
     <t>Wafers горіх ВКФ 216г /16шт</t>
   </si>
   <si>
-    <t>Wafers горіх ВКФ 72г /22шт AR /</t>
-  </si>
-  <si>
     <t>Wafers горіх ККФ 216г /16шт</t>
   </si>
   <si>
+    <t>Wafers горіх ККФ 216г /16шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Wafers какао ККФ 216г /16шт</t>
   </si>
   <si>
+    <t>Wafers какао ККФ 216г /16шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Wafers какао ККФ 72г /22шт AR /</t>
   </si>
   <si>
     <t>Wafers какао-молоко ККФ 216г /16шт</t>
   </si>
   <si>
+    <t>Wafers какао-молоко ККФ 216г /16шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Wafers кокос та мигдаль ВКФ 216г /16шт</t>
   </si>
   <si>
-    <t>Wafers лимон ВКФ 216г /16шт</t>
+    <t>Wafers кокос та мигдаль ВКФ 216г /16шт АКЦІЯ Цінова</t>
   </si>
   <si>
     <t>Wafers лимон ВКФ 72г /22шт AR /</t>
   </si>
   <si>
-    <t>Wafers лимон ККФ 216г /16шт</t>
+    <t>Wafers лимон ККФ 216г /16шт АКЦІЯ Цінова</t>
   </si>
   <si>
     <t>Wafers молоко ВКФ 216г /16шт</t>
   </si>
   <si>
+    <t>Wafers молоко ВКФ 216г /16шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Wafers молоко ВКФ 72г /22шт AR /</t>
   </si>
   <si>
@@ -458,6 +482,9 @@
     <t>Bonny-Fruit літній мікс ВКФ 200г /18шт /</t>
   </si>
   <si>
+    <t>Bonny-Fruit цитрусовий мікс ВКФ 200г /18шт /</t>
+  </si>
+  <si>
     <t>Bonny-Fruit ягідний мікс ВКФ 200г /18шт /</t>
   </si>
   <si>
@@ -479,6 +506,9 @@
     <t>Yummi Gummi Apples ВКФ 165г /14шт</t>
   </si>
   <si>
+    <t>Yummi Gummi Apples ВКФ 165г /14шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Yummi Gummi Apples ВКФ 165г /14шт АКЦІЯ Цінова</t>
   </si>
   <si>
@@ -518,9 +548,6 @@
     <t>Yummi Gummi Daydream ВКФ 70г /22шт АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Yummi Gummi Daydream ВКФ 70г /22шт АКЦІЯ Цінова TP</t>
-  </si>
-  <si>
     <t>Yummi Gummi Donuts ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -533,21 +560,12 @@
     <t>Yummi Gummi Duo Mix ВКФ 70г /22шт АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Yummi Gummi Duo Mix ВКФ 70г /22шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
-    <t>Yummi Gummi Duo Mix ВКФ 70г /22шт АКЦІЯ Цінова TP</t>
-  </si>
-  <si>
     <t>Yummi Gummi Fizzy Worms ВКФ 70г /22шт</t>
   </si>
   <si>
     <t>Yummi Gummi Fizzy Worms ВКФ 70г /22шт АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Yummi Gummi Fizzy Worms ВКФ 70г /22шт АКЦІЯ Цінова накладна TP</t>
-  </si>
-  <si>
     <t>Yummi Gummi Fluffi Barbecue ВКФ 200г /7шт</t>
   </si>
   <si>
@@ -617,7 +635,7 @@
     <t>Yummi Gummi Mini Bear Mix ВКФ 70г /22шт АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Yummi Gummi Mini Bear Mix ВКФ 70г /22шт АКЦІЯ Цінова накладна TP</t>
+    <t>Yummi Gummi Mini Bear Mix ВКФ 70г /22шт АКЦІЯ Цінова TP</t>
   </si>
   <si>
     <t>Yummi Gummi Pasta ВКФ 70г /22шт</t>
@@ -626,9 +644,15 @@
     <t>Yummi Gummi Pasta ВКФ 70г /22шт АКЦІЯ ОПТ</t>
   </si>
   <si>
+    <t>Yummi Gummi Rabbits ВКФ 165г /14шт</t>
+  </si>
+  <si>
     <t>Yummi Gummi Rabbits ВКФ 165г /14шт АКЦІЯ ВІП</t>
   </si>
   <si>
+    <t>Yummi Gummi Rainbow Wands ВКФ 165г /14шт</t>
+  </si>
+  <si>
     <t>Yummi Gummi Rainbow Wands ВКФ 165г /14шт АКЦІЯ ВІП</t>
   </si>
   <si>
@@ -644,24 +668,21 @@
     <t>Yummi Gummi Sour Belts ВКФ 70г /40шт АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Yummi Gummi Sour Belts ВКФ 70г /40шт АКЦІЯ Цінова</t>
-  </si>
-  <si>
-    <t>Yummi Gummi Sour Belts ВКФ 70г /40шт АКЦІЯ Цінова TP</t>
-  </si>
-  <si>
     <t>Yummi Gummi Sour Belts ВКФ 70г /40шт АКЦІЯ Цінова накладна</t>
   </si>
   <si>
+    <t>Yummi Gummi Sour Slices ВКФ 165г /14шт</t>
+  </si>
+  <si>
+    <t>Yummi Gummi Sour Slices ВКФ 165г /14шт АКЦІЯ ВІП</t>
+  </si>
+  <si>
     <t>Yummi Gummi Sour Sticks ВКФ 70г /40шт</t>
   </si>
   <si>
     <t>Yummi Gummi Sour Sticks ВКФ 70г /40шт АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Yummi Gummi Sour Sticks ВКФ 70г /40шт АКЦІЯ Цінова TP</t>
-  </si>
-  <si>
     <t>Yummi Gummi Sour Strawberries ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -677,9 +698,6 @@
     <t>Yummi Gummi Twists ВКФ 70г /40шт АКЦІЯ ОПТ</t>
   </si>
   <si>
-    <t>Yummi Gummi Twists ВКФ 70г /40шт АКЦІЯ Цінова TP</t>
-  </si>
-  <si>
     <t>Yummi Gummi Watermelon Slices ВКФ 70г /22шт</t>
   </si>
   <si>
@@ -740,9 +758,6 @@
     <t>Lollipops GUM Фруктовий мікс РЦ 0.92кг /9шт</t>
   </si>
   <si>
-    <t>LolliPops з йогуртовими смаками РЦ 0.92кг /9шт</t>
-  </si>
-  <si>
     <t>LolliPops з коктельними смаками РЦ 0.92кг /9шт /</t>
   </si>
   <si>
@@ -770,9 +785,6 @@
     <t>Roshen Yogurtini РЦ 1кг /8шт</t>
   </si>
   <si>
-    <t>Toffelini з какао-начинкою ВКФ 1кг /6пак</t>
-  </si>
-  <si>
     <t>Yummi's РЦ 1кг /7пак</t>
   </si>
   <si>
@@ -812,6 +824,9 @@
     <t>Шалена бджілка ВКФ 1кг /9пак</t>
   </si>
   <si>
+    <t>Шалена бджілка ВКФ 1кг /9пак АКЦІЯ</t>
+  </si>
+  <si>
     <t>Шипучка РЦ 1кг /7пак</t>
   </si>
   <si>
@@ -836,6 +851,9 @@
     <t>Cherry Queen heart РЦ 122г /8шт АКЦІЯ ВІП</t>
   </si>
   <si>
+    <t>Chocolateria ВКФ 194г /8шт NEW</t>
+  </si>
+  <si>
     <t>Chocolateria ВКФ 256г /8шт</t>
   </si>
   <si>
@@ -899,6 +917,12 @@
     <t>Lovita Cake Cookies з яблуком та корицею ККФ 168г /16шт</t>
   </si>
   <si>
+    <t>Lovita Classic Cookies арахіс ККФ 150г /16шт</t>
+  </si>
+  <si>
+    <t>Lovita Classic Cookies з какао і кусочками глазурі ККФ 150г /16шт</t>
+  </si>
+  <si>
     <t>Lovita Classic Cookies з кусочками глазурі ВКФ 150г /16шт</t>
   </si>
   <si>
@@ -914,12 +938,12 @@
     <t>Lovita Jelly Cookies з желейною начинкою зі смаком полуниці ККФ 135г /21шт /</t>
   </si>
   <si>
-    <t>Lovita Jelly Cookies з желейною начинкою зі смаком полуниці ККФ 420г /7шт</t>
-  </si>
-  <si>
     <t>Lovita Jelly Cookies з желейною начинкою какао + вишня ККФ 135г /21шт /</t>
   </si>
   <si>
+    <t>Lovita Jelly Cookies з желейною начинкою какао + вишня ККФ 420г /7шт</t>
+  </si>
+  <si>
     <t>Lovita Soft Cream Cookies cocoa ККФ 127г /18шт</t>
   </si>
   <si>
@@ -947,9 +971,6 @@
     <t>Multicake з начинкою кокос-крем ККФ 180г /28шт FP</t>
   </si>
   <si>
-    <t>Multicake з начинкою лимон-крем ККФ 180г /28шт FP</t>
-  </si>
-  <si>
     <t>Multicake з начинкою полуниця-крем ККФ 180г /28шт FP</t>
   </si>
   <si>
@@ -980,6 +1001,9 @@
     <t>Candy Nut м'яка карамель з арахісом ВКФ 1кг /8пак PT ЗНИЖКА ДИСТР</t>
   </si>
   <si>
+    <t>Candy Nut нуга і м'яка карамель з арахісом ВКФ 1кг /5пак ЗНИЖКА ДИСТР</t>
+  </si>
+  <si>
     <t>Candy Nut нуга карамель арахіс 1кг/5</t>
   </si>
   <si>
@@ -995,16 +1019,19 @@
     <t>Johnny Krocker choco ВКФ 1кг /4шт PL</t>
   </si>
   <si>
-    <t>Johnny Krocker coconut ВКФ 1кг /4шт</t>
+    <t>Johnny Krocker choco ВКФ 1кг /4шт ЗНИЖКА ДИСТР</t>
+  </si>
+  <si>
+    <t>Johnny Krocker coconut ВКФ 1кг /4шт ЗНИЖКА ДИСТР</t>
   </si>
   <si>
     <t>Johnny Krocker milk ВКФ 1кг /4шт PL</t>
   </si>
   <si>
-    <t>KONAFETTO blanc ККФ 1кг /5пак HAL</t>
-  </si>
-  <si>
-    <t>KONAFETTO nero ККФ 1кг /5пак HAL</t>
+    <t>Johnny Krocker milk ВКФ 1кг /4шт ЗНИЖКА ДИСТР</t>
+  </si>
+  <si>
+    <t>Ko-Ko Choco White 1кг/5</t>
   </si>
   <si>
     <t>Krock з арахісовою пастою ВКФ 1кг /8пак</t>
@@ -1034,12 +1061,6 @@
     <t>Монблан з мигдалем та кокосовим кремом ВКФ 1кг /4пак ЗНИЖКА ДИСТР</t>
   </si>
   <si>
-    <t>Монблан з подр. мигдалем та кокосовим кремом ВКФ 1кг /4пак</t>
-  </si>
-  <si>
-    <t>Монблан з подрібненим мигдалем ВКФ 1кг /4пак</t>
-  </si>
-  <si>
     <t>Монблан з подрібненим мигдалем ВКФ 1кг /4пак ЗНИЖКА ДИСТР</t>
   </si>
   <si>
@@ -1082,6 +1103,9 @@
     <t>Червоний мак ВКФ 1кг /7пак</t>
   </si>
   <si>
+    <t>Червоний мак ВКФ 1кг /7пак АКЦІЯ ВІП 1</t>
+  </si>
+  <si>
     <t>Шоколапки ВКФ 1кг /7пак</t>
   </si>
   <si>
@@ -1097,9 +1121,6 @@
     <t>ШОКОЛАД</t>
   </si>
   <si>
-    <t>Lacmi Big Bite молочний ВКФ 200г /17шт</t>
-  </si>
-  <si>
     <t>Lacmi Big Bite молочний ВКФ 200г /17шт АКЦІЯ Цінова</t>
   </si>
   <si>
@@ -1127,9 +1148,6 @@
     <t>Lacmi Fun&amp;Crispy молочний пористий з молочною начинкою з кріспі ВКФ 85г /17шт</t>
   </si>
   <si>
-    <t>Lacmi Fun&amp;Crispy молочний пористий з молочною начинкою з кріспі ВКФ 85г /17шт АКЦІЯ Цінова UA</t>
-  </si>
-  <si>
     <t>Lacmi молочний Strawberry cake ВКФ 275г /12шт</t>
   </si>
   <si>
@@ -1229,24 +1247,48 @@
     <t>Roshen Nut молочний з цілим мигдалем ВКФ 90г /20шт</t>
   </si>
   <si>
+    <t>Roshen Nut молочний з цілим мигдалем ВКФ 90г /20шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Roshen Nut молочний з цілим фундуком ВКФ 90г /18шт</t>
   </si>
   <si>
+    <t>Roshen Nut молочний з цілим фундуком ВКФ 90г /18шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Roshen Nut чорний з цілим мигдалем ВКФ 90г /20шт</t>
   </si>
   <si>
+    <t>Roshen Nut чорний з цілим мигдалем ВКФ 90г /20шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
     <t>Roshen Nut чорний з цілим фундуком ВКФ 90г /18шт</t>
   </si>
   <si>
+    <t>Roshen Nut чорний з цілим фундуком ВКФ 90г /18шт АКЦІЯ Цінова</t>
+  </si>
+  <si>
+    <t>Roshen пористий БІЛИЙ ВКФ 80г /20шт Aerated АКЦІЯ Цінова UA</t>
+  </si>
+  <si>
     <t>Roshen пористий білий карамельний ВКФ 80г /20шт Aerated UA</t>
   </si>
   <si>
+    <t>Roshen пористий білий карамельний ВКФ 80г /20шт Aerated АКЦІЯ Цінова UA</t>
+  </si>
+  <si>
     <t>Roshen пористий екстрачорний ВКФ 80г /20шт Aerated UA</t>
   </si>
   <si>
+    <t>Roshen пористий екстрачорний ВКФ 80г /20шт Aerated АКЦІЯ Цінова UA</t>
+  </si>
+  <si>
     <t>Roshen пористий молочний ВКФ 80г /20шт Aerated UA</t>
   </si>
   <si>
+    <t>Roshen пористий молочний ВКФ 80г /20шт Aerated АКЦІЯ Цінова UA</t>
+  </si>
+  <si>
     <t>Roshen чорний Bitter 80% ВКФ 85г /35шт</t>
   </si>
   <si>
@@ -1268,10 +1310,10 @@
     <t>ФІГУРКИ</t>
   </si>
   <si>
-    <t>Кролик Roshen весняний ВКФ 25г /35шт</t>
-  </si>
-  <si>
     <t>Кролик Roshen весняний ВКФ 25г /35шт АКЦІЯ</t>
+  </si>
+  <si>
+    <t>Кролик Roshen весняний ВКФ 25г /35шт АКЦІЯ ВІП</t>
   </si>
   <si>
     <t>Кролик Roshen весняний ВКФ 40г /24шт</t>
@@ -1529,7 +1571,7 @@
     <outlinePr summaryBelow="false" summaryRight="false"/>
     <pageSetUpPr autoPageBreaks="false"/>
   </sheetPr>
-  <dimension ref="C420"/>
+  <dimension ref="C434"/>
   <sheetFormatPr defaultColWidth="10.5" customHeight="true" defaultRowHeight="11.429"/>
   <cols>
     <col min="1" max="1" width="2.33203125" style="1" customWidth="true"/>
@@ -1594,7 +1636,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>129</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" ht="11" customHeight="true">
@@ -1602,7 +1644,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="12" t="n">
-        <v>181087</v>
+        <v>156794</v>
       </c>
     </row>
     <row r="13" ht="11" customHeight="true" outlineLevel="1">
@@ -1610,7 +1652,7 @@
         <v>12</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>35859</v>
+        <v>44418</v>
       </c>
     </row>
     <row r="14" ht="11" customHeight="true" outlineLevel="2">
@@ -1618,7 +1660,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>6678</v>
+        <v>4054</v>
       </c>
     </row>
     <row r="15" ht="11" customHeight="true" outlineLevel="3">
@@ -1626,15 +1668,15 @@
         <v>14</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>720</v>
+        <v>600</v>
       </c>
     </row>
     <row r="16" ht="11" customHeight="true" outlineLevel="3">
       <c r="B16" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="16" t="n">
-        <v>1696</v>
+      <c r="C16" s="11" t="n">
+        <v>308</v>
       </c>
     </row>
     <row r="17" ht="11" customHeight="true" outlineLevel="3">
@@ -1642,7 +1684,7 @@
         <v>16</v>
       </c>
       <c r="C17" s="11" t="n">
-        <v>320</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" ht="11" customHeight="true" outlineLevel="3">
@@ -1650,7 +1692,7 @@
         <v>17</v>
       </c>
       <c r="C18" s="11" t="n">
-        <v>32</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" ht="11" customHeight="true" outlineLevel="3">
@@ -1658,7 +1700,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="11" t="n">
-        <v>298</v>
+        <v>377</v>
       </c>
     </row>
     <row r="20" ht="11" customHeight="true" outlineLevel="3">
@@ -1666,7 +1708,7 @@
         <v>19</v>
       </c>
       <c r="C20" s="11" t="n">
-        <v>977</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" ht="11" customHeight="true" outlineLevel="3">
@@ -1682,7 +1724,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>340</v>
+        <v>492</v>
       </c>
     </row>
     <row r="23" ht="11" customHeight="true" outlineLevel="3">
@@ -1690,23 +1732,23 @@
         <v>22</v>
       </c>
       <c r="C23" s="11" t="n">
-        <v>275</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" ht="11" customHeight="true" outlineLevel="3">
       <c r="B24" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C24" s="16" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="25" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B25" s="14" t="s">
+      <c r="C24" s="11" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="25" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B25" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C25" s="12" t="n">
-        <v>15273</v>
+      <c r="C25" s="11" t="n">
+        <v>405</v>
       </c>
     </row>
     <row r="26" ht="11" customHeight="true" outlineLevel="3">
@@ -1714,15 +1756,15 @@
         <v>25</v>
       </c>
       <c r="C26" s="16" t="n">
-        <v>1090</v>
-      </c>
-    </row>
-    <row r="27" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B27" s="15" t="s">
+        <v>1414</v>
+      </c>
+    </row>
+    <row r="27" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B27" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="16" t="n">
-        <v>1188</v>
+      <c r="C27" s="12" t="n">
+        <v>19243</v>
       </c>
     </row>
     <row r="28" ht="11" customHeight="true" outlineLevel="3">
@@ -1730,7 +1772,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>210</v>
+        <v>999</v>
       </c>
     </row>
     <row r="29" ht="11" customHeight="true" outlineLevel="3">
@@ -1738,7 +1780,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="11" t="n">
-        <v>556</v>
+        <v>436</v>
       </c>
     </row>
     <row r="30" ht="11" customHeight="true" outlineLevel="3">
@@ -1746,7 +1788,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>52</v>
+        <v>380</v>
       </c>
     </row>
     <row r="31" ht="11" customHeight="true" outlineLevel="3">
@@ -1754,15 +1796,15 @@
         <v>30</v>
       </c>
       <c r="C31" s="11" t="n">
-        <v>595</v>
+        <v>12</v>
       </c>
     </row>
     <row r="32" ht="11" customHeight="true" outlineLevel="3">
       <c r="B32" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="C32" s="16" t="n">
-        <v>1048</v>
+      <c r="C32" s="11" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="33" ht="11" customHeight="true" outlineLevel="3">
@@ -1778,23 +1820,23 @@
         <v>33</v>
       </c>
       <c r="C34" s="16" t="n">
-        <v>2015</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="35" ht="11" customHeight="true" outlineLevel="3">
       <c r="B35" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>815</v>
+      <c r="C35" s="16" t="n">
+        <v>1490</v>
       </c>
     </row>
     <row r="36" ht="11" customHeight="true" outlineLevel="3">
       <c r="B36" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>990</v>
+      <c r="C36" s="16" t="n">
+        <v>2778</v>
       </c>
     </row>
     <row r="37" ht="11" customHeight="true" outlineLevel="3">
@@ -1802,7 +1844,7 @@
         <v>36</v>
       </c>
       <c r="C37" s="16" t="n">
-        <v>1222</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="38" ht="11" customHeight="true" outlineLevel="3">
@@ -1810,31 +1852,31 @@
         <v>37</v>
       </c>
       <c r="C38" s="16" t="n">
-        <v>4784</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="39" ht="11" customHeight="true" outlineLevel="3">
       <c r="B39" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C39" s="11" t="n">
-        <v>21</v>
+      <c r="C39" s="16" t="n">
+        <v>2350</v>
       </c>
     </row>
     <row r="40" ht="11" customHeight="true" outlineLevel="3">
       <c r="B40" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C40" s="11" t="n">
-        <v>64</v>
+      <c r="C40" s="16" t="n">
+        <v>1891</v>
       </c>
     </row>
     <row r="41" ht="11" customHeight="true" outlineLevel="3">
       <c r="B41" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="C41" s="11" t="n">
-        <v>334</v>
+      <c r="C41" s="16" t="n">
+        <v>2050</v>
       </c>
     </row>
     <row r="42" ht="11" customHeight="true" outlineLevel="3">
@@ -1842,7 +1884,7 @@
         <v>41</v>
       </c>
       <c r="C42" s="11" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
     </row>
     <row r="43" ht="11" customHeight="true" outlineLevel="3">
@@ -1850,7 +1892,7 @@
         <v>42</v>
       </c>
       <c r="C43" s="11" t="n">
-        <v>61</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" ht="11" customHeight="true" outlineLevel="3">
@@ -1858,7 +1900,7 @@
         <v>43</v>
       </c>
       <c r="C44" s="11" t="n">
-        <v>88</v>
+        <v>334</v>
       </c>
     </row>
     <row r="45" ht="11" customHeight="true" outlineLevel="3">
@@ -1866,15 +1908,15 @@
         <v>44</v>
       </c>
       <c r="C45" s="11" t="n">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="46" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B46" s="14" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B46" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C46" s="12" t="n">
-        <v>5840</v>
+      <c r="C46" s="11" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="47" ht="11" customHeight="true" outlineLevel="3">
@@ -1882,7 +1924,7 @@
         <v>46</v>
       </c>
       <c r="C47" s="11" t="n">
-        <v>363</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48" ht="11" customHeight="true" outlineLevel="3">
@@ -1890,15 +1932,15 @@
         <v>47</v>
       </c>
       <c r="C48" s="11" t="n">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="49" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B49" s="15" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="49" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B49" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C49" s="11" t="n">
-        <v>423</v>
+      <c r="C49" s="12" t="n">
+        <v>5456</v>
       </c>
     </row>
     <row r="50" ht="11" customHeight="true" outlineLevel="3">
@@ -1906,7 +1948,7 @@
         <v>49</v>
       </c>
       <c r="C50" s="11" t="n">
-        <v>46</v>
+        <v>212</v>
       </c>
     </row>
     <row r="51" ht="11" customHeight="true" outlineLevel="3">
@@ -1914,7 +1956,7 @@
         <v>50</v>
       </c>
       <c r="C51" s="11" t="n">
-        <v>7</v>
+        <v>272</v>
       </c>
     </row>
     <row r="52" ht="11" customHeight="true" outlineLevel="3">
@@ -1922,7 +1964,7 @@
         <v>51</v>
       </c>
       <c r="C52" s="11" t="n">
-        <v>276</v>
+        <v>82</v>
       </c>
     </row>
     <row r="53" ht="11" customHeight="true" outlineLevel="3">
@@ -1930,7 +1972,7 @@
         <v>52</v>
       </c>
       <c r="C53" s="11" t="n">
-        <v>156</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54" ht="11" customHeight="true" outlineLevel="3">
@@ -1938,7 +1980,7 @@
         <v>53</v>
       </c>
       <c r="C54" s="11" t="n">
-        <v>170</v>
+        <v>232</v>
       </c>
     </row>
     <row r="55" ht="11" customHeight="true" outlineLevel="3">
@@ -1946,7 +1988,7 @@
         <v>54</v>
       </c>
       <c r="C55" s="11" t="n">
-        <v>126</v>
+        <v>240</v>
       </c>
     </row>
     <row r="56" ht="11" customHeight="true" outlineLevel="3">
@@ -1954,7 +1996,7 @@
         <v>55</v>
       </c>
       <c r="C56" s="11" t="n">
-        <v>592</v>
+        <v>81</v>
       </c>
     </row>
     <row r="57" ht="11" customHeight="true" outlineLevel="3">
@@ -1962,7 +2004,7 @@
         <v>56</v>
       </c>
       <c r="C57" s="11" t="n">
-        <v>911</v>
+        <v>108</v>
       </c>
     </row>
     <row r="58" ht="11" customHeight="true" outlineLevel="3">
@@ -1970,7 +2012,7 @@
         <v>57</v>
       </c>
       <c r="C58" s="11" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
     </row>
     <row r="59" ht="11" customHeight="true" outlineLevel="3">
@@ -1978,7 +2020,7 @@
         <v>58</v>
       </c>
       <c r="C59" s="11" t="n">
-        <v>96</v>
+        <v>475</v>
       </c>
     </row>
     <row r="60" ht="11" customHeight="true" outlineLevel="3">
@@ -1986,7 +2028,7 @@
         <v>59</v>
       </c>
       <c r="C60" s="11" t="n">
-        <v>234</v>
+        <v>262</v>
       </c>
     </row>
     <row r="61" ht="11" customHeight="true" outlineLevel="3">
@@ -1994,7 +2036,7 @@
         <v>60</v>
       </c>
       <c r="C61" s="11" t="n">
-        <v>177</v>
+        <v>476</v>
       </c>
     </row>
     <row r="62" ht="11" customHeight="true" outlineLevel="3">
@@ -2002,7 +2044,7 @@
         <v>61</v>
       </c>
       <c r="C62" s="11" t="n">
-        <v>458</v>
+        <v>116</v>
       </c>
     </row>
     <row r="63" ht="11" customHeight="true" outlineLevel="3">
@@ -2010,7 +2052,7 @@
         <v>62</v>
       </c>
       <c r="C63" s="11" t="n">
-        <v>18</v>
+        <v>289</v>
       </c>
     </row>
     <row r="64" ht="11" customHeight="true" outlineLevel="3">
@@ -2018,23 +2060,23 @@
         <v>63</v>
       </c>
       <c r="C64" s="11" t="n">
-        <v>30</v>
+        <v>96</v>
       </c>
     </row>
     <row r="65" ht="11" customHeight="true" outlineLevel="3">
       <c r="B65" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="C65" s="16" t="n">
-        <v>1475</v>
-      </c>
-    </row>
-    <row r="66" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B66" s="14" t="s">
+      <c r="C65" s="11" t="n">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B66" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="C66" s="12" t="n">
-        <v>8068</v>
+      <c r="C66" s="11" t="n">
+        <v>120</v>
       </c>
     </row>
     <row r="67" ht="11" customHeight="true" outlineLevel="3">
@@ -2042,7 +2084,7 @@
         <v>66</v>
       </c>
       <c r="C67" s="11" t="n">
-        <v>87</v>
+        <v>268</v>
       </c>
     </row>
     <row r="68" ht="11" customHeight="true" outlineLevel="3">
@@ -2050,7 +2092,7 @@
         <v>67</v>
       </c>
       <c r="C68" s="11" t="n">
-        <v>238</v>
+        <v>80</v>
       </c>
     </row>
     <row r="69" ht="11" customHeight="true" outlineLevel="3">
@@ -2058,7 +2100,7 @@
         <v>68</v>
       </c>
       <c r="C69" s="11" t="n">
-        <v>84</v>
+        <v>18</v>
       </c>
     </row>
     <row r="70" ht="11" customHeight="true" outlineLevel="3">
@@ -2066,23 +2108,23 @@
         <v>69</v>
       </c>
       <c r="C70" s="11" t="n">
-        <v>406</v>
+        <v>22</v>
       </c>
     </row>
     <row r="71" ht="11" customHeight="true" outlineLevel="3">
       <c r="B71" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="C71" s="11" t="n">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="72" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B72" s="15" t="s">
+      <c r="C71" s="16" t="n">
+        <v>1332</v>
+      </c>
+    </row>
+    <row r="72" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B72" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C72" s="11" t="n">
-        <v>270</v>
+      <c r="C72" s="12" t="n">
+        <v>15665</v>
       </c>
     </row>
     <row r="73" ht="11" customHeight="true" outlineLevel="3">
@@ -2090,7 +2132,7 @@
         <v>72</v>
       </c>
       <c r="C73" s="11" t="n">
-        <v>398</v>
+        <v>148</v>
       </c>
     </row>
     <row r="74" ht="11" customHeight="true" outlineLevel="3">
@@ -2098,7 +2140,7 @@
         <v>73</v>
       </c>
       <c r="C74" s="11" t="n">
-        <v>456</v>
+        <v>308</v>
       </c>
     </row>
     <row r="75" ht="11" customHeight="true" outlineLevel="3">
@@ -2106,7 +2148,7 @@
         <v>74</v>
       </c>
       <c r="C75" s="11" t="n">
-        <v>10</v>
+        <v>55</v>
       </c>
     </row>
     <row r="76" ht="11" customHeight="true" outlineLevel="3">
@@ -2114,7 +2156,7 @@
         <v>75</v>
       </c>
       <c r="C76" s="11" t="n">
-        <v>441</v>
+        <v>227</v>
       </c>
     </row>
     <row r="77" ht="11" customHeight="true" outlineLevel="3">
@@ -2122,7 +2164,7 @@
         <v>76</v>
       </c>
       <c r="C77" s="11" t="n">
-        <v>331</v>
+        <v>889</v>
       </c>
     </row>
     <row r="78" ht="11" customHeight="true" outlineLevel="3">
@@ -2130,15 +2172,15 @@
         <v>77</v>
       </c>
       <c r="C78" s="11" t="n">
-        <v>889</v>
+        <v>681</v>
       </c>
     </row>
     <row r="79" ht="11" customHeight="true" outlineLevel="3">
       <c r="B79" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C79" s="16" t="n">
-        <v>3342</v>
+      <c r="C79" s="11" t="n">
+        <v>771</v>
       </c>
     </row>
     <row r="80" ht="11" customHeight="true" outlineLevel="3">
@@ -2146,7 +2188,7 @@
         <v>79</v>
       </c>
       <c r="C80" s="11" t="n">
-        <v>319</v>
+        <v>238</v>
       </c>
     </row>
     <row r="81" ht="11" customHeight="true" outlineLevel="3">
@@ -2154,39 +2196,39 @@
         <v>80</v>
       </c>
       <c r="C81" s="11" t="n">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="82" ht="11" customHeight="true" outlineLevel="1">
-      <c r="B82" s="13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="82" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B82" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C82" s="12" t="n">
-        <v>145228</v>
-      </c>
-    </row>
-    <row r="83" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B83" s="14" t="s">
+      <c r="C82" s="11" t="n">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="83" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B83" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="C83" s="12" t="n">
-        <v>42330</v>
-      </c>
-    </row>
-    <row r="84" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C83" s="16" t="n">
+        <v>1093</v>
+      </c>
+    </row>
+    <row r="84" ht="11" customHeight="true" outlineLevel="3">
       <c r="B84" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="C84" s="16" t="n">
-        <v>2315</v>
-      </c>
-    </row>
-    <row r="85" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C84" s="11" t="n">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="85" ht="11" customHeight="true" outlineLevel="3">
       <c r="B85" s="15" t="s">
         <v>84</v>
       </c>
       <c r="C85" s="16" t="n">
-        <v>5518</v>
+        <v>10526</v>
       </c>
     </row>
     <row r="86" ht="11" customHeight="true" outlineLevel="3">
@@ -2194,31 +2236,31 @@
         <v>85</v>
       </c>
       <c r="C86" s="11" t="n">
-        <v>964</v>
-      </c>
-    </row>
-    <row r="87" ht="22" customHeight="true" outlineLevel="3">
-      <c r="B87" s="15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="87" ht="11" customHeight="true" outlineLevel="1">
+      <c r="B87" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="C87" s="16" t="n">
-        <v>1049</v>
-      </c>
-    </row>
-    <row r="88" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B88" s="15" t="s">
+      <c r="C87" s="12" t="n">
+        <v>112376</v>
+      </c>
+    </row>
+    <row r="88" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B88" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="C88" s="11" t="n">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="89" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C88" s="12" t="n">
+        <v>25516</v>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="true" outlineLevel="3">
       <c r="B89" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="C89" s="16" t="n">
-        <v>1680</v>
+      <c r="C89" s="11" t="n">
+        <v>365</v>
       </c>
     </row>
     <row r="90" ht="22" customHeight="true" outlineLevel="3">
@@ -2226,7 +2268,7 @@
         <v>89</v>
       </c>
       <c r="C90" s="11" t="n">
-        <v>360</v>
+        <v>900</v>
       </c>
     </row>
     <row r="91" ht="22" customHeight="true" outlineLevel="3">
@@ -2234,55 +2276,55 @@
         <v>90</v>
       </c>
       <c r="C91" s="16" t="n">
-        <v>2835</v>
-      </c>
-    </row>
-    <row r="92" ht="22" customHeight="true" outlineLevel="3">
+        <v>3928</v>
+      </c>
+    </row>
+    <row r="92" ht="11" customHeight="true" outlineLevel="3">
       <c r="B92" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="C92" s="16" t="n">
-        <v>5100</v>
+      <c r="C92" s="11" t="n">
+        <v>394</v>
       </c>
     </row>
     <row r="93" ht="22" customHeight="true" outlineLevel="3">
       <c r="B93" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="C93" s="16" t="n">
-        <v>2400</v>
-      </c>
-    </row>
-    <row r="94" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C93" s="11" t="n">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="94" ht="11" customHeight="true" outlineLevel="3">
       <c r="B94" s="15" t="s">
         <v>93</v>
       </c>
       <c r="C94" s="16" t="n">
-        <v>4005</v>
-      </c>
-    </row>
-    <row r="95" ht="22" customHeight="true" outlineLevel="3">
+        <v>1110</v>
+      </c>
+    </row>
+    <row r="95" ht="11" customHeight="true" outlineLevel="3">
       <c r="B95" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="C95" s="16" t="n">
-        <v>2488</v>
+      <c r="C95" s="11" t="n">
+        <v>900</v>
       </c>
     </row>
     <row r="96" ht="22" customHeight="true" outlineLevel="3">
       <c r="B96" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="C96" s="16" t="n">
-        <v>5029</v>
+      <c r="C96" s="11" t="n">
+        <v>360</v>
       </c>
     </row>
     <row r="97" ht="22" customHeight="true" outlineLevel="3">
       <c r="B97" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="C97" s="11" t="n">
-        <v>20</v>
+      <c r="C97" s="16" t="n">
+        <v>1575</v>
       </c>
     </row>
     <row r="98" ht="22" customHeight="true" outlineLevel="3">
@@ -2290,7 +2332,7 @@
         <v>97</v>
       </c>
       <c r="C98" s="11" t="n">
-        <v>150</v>
+        <v>180</v>
       </c>
     </row>
     <row r="99" ht="22" customHeight="true" outlineLevel="3">
@@ -2298,7 +2340,7 @@
         <v>98</v>
       </c>
       <c r="C99" s="16" t="n">
-        <v>2884</v>
+        <v>3477</v>
       </c>
     </row>
     <row r="100" ht="22" customHeight="true" outlineLevel="3">
@@ -2306,95 +2348,95 @@
         <v>99</v>
       </c>
       <c r="C100" s="16" t="n">
-        <v>4277</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="101" ht="22" customHeight="true" outlineLevel="3">
       <c r="B101" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="C101" s="16" t="n">
-        <v>1003</v>
-      </c>
-    </row>
-    <row r="102" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B102" s="14" t="s">
+      <c r="C101" s="11" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B102" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="C102" s="12" t="n">
-        <v>1321</v>
-      </c>
-    </row>
-    <row r="103" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C102" s="16" t="n">
+        <v>2055</v>
+      </c>
+    </row>
+    <row r="103" ht="22" customHeight="true" outlineLevel="3">
       <c r="B103" s="15" t="s">
         <v>102</v>
       </c>
       <c r="C103" s="11" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="104" ht="11" customHeight="true" outlineLevel="3">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="true" outlineLevel="3">
       <c r="B104" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="C104" s="11" t="n">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="105" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C104" s="16" t="n">
+        <v>2929</v>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="true" outlineLevel="3">
       <c r="B105" s="15" t="s">
         <v>104</v>
       </c>
       <c r="C105" s="11" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="106" ht="11" customHeight="true" outlineLevel="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="true" outlineLevel="3">
       <c r="B106" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="C106" s="11" t="n">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="107" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C106" s="16" t="n">
+        <v>1143</v>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="true" outlineLevel="3">
       <c r="B107" s="15" t="s">
         <v>106</v>
       </c>
       <c r="C107" s="11" t="n">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="108" ht="11" customHeight="true" outlineLevel="3">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="true" outlineLevel="3">
       <c r="B108" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="C108" s="11" t="n">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="109" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C108" s="16" t="n">
+        <v>1815</v>
+      </c>
+    </row>
+    <row r="109" ht="22" customHeight="true" outlineLevel="3">
       <c r="B109" s="15" t="s">
         <v>108</v>
       </c>
       <c r="C109" s="11" t="n">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="110" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B110" s="15" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="110" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B110" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C110" s="11" t="n">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="111" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B111" s="14" t="s">
+      <c r="C110" s="12" t="n">
+        <v>3246</v>
+      </c>
+    </row>
+    <row r="111" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B111" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="C111" s="12" t="n">
-        <v>29896</v>
+      <c r="C111" s="11" t="n">
+        <v>397</v>
       </c>
     </row>
     <row r="112" ht="11" customHeight="true" outlineLevel="3">
@@ -2402,7 +2444,7 @@
         <v>111</v>
       </c>
       <c r="C112" s="11" t="n">
-        <v>92</v>
+        <v>505</v>
       </c>
     </row>
     <row r="113" ht="11" customHeight="true" outlineLevel="3">
@@ -2410,7 +2452,7 @@
         <v>112</v>
       </c>
       <c r="C113" s="11" t="n">
-        <v>24</v>
+        <v>778</v>
       </c>
     </row>
     <row r="114" ht="11" customHeight="true" outlineLevel="3">
@@ -2418,7 +2460,7 @@
         <v>113</v>
       </c>
       <c r="C114" s="11" t="n">
-        <v>204</v>
+        <v>475</v>
       </c>
     </row>
     <row r="115" ht="11" customHeight="true" outlineLevel="3">
@@ -2426,7 +2468,7 @@
         <v>114</v>
       </c>
       <c r="C115" s="11" t="n">
-        <v>86</v>
+        <v>249</v>
       </c>
     </row>
     <row r="116" ht="11" customHeight="true" outlineLevel="3">
@@ -2434,39 +2476,39 @@
         <v>115</v>
       </c>
       <c r="C116" s="11" t="n">
-        <v>136</v>
+        <v>311</v>
       </c>
     </row>
     <row r="117" ht="11" customHeight="true" outlineLevel="3">
       <c r="B117" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="C117" s="16" t="n">
-        <v>9975</v>
+      <c r="C117" s="11" t="n">
+        <v>87</v>
       </c>
     </row>
     <row r="118" ht="11" customHeight="true" outlineLevel="3">
       <c r="B118" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="C118" s="16" t="n">
-        <v>11297</v>
+      <c r="C118" s="11" t="n">
+        <v>245</v>
       </c>
     </row>
     <row r="119" ht="11" customHeight="true" outlineLevel="3">
       <c r="B119" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="C119" s="16" t="n">
-        <v>1700</v>
-      </c>
-    </row>
-    <row r="120" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B120" s="15" t="s">
+      <c r="C119" s="11" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="120" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B120" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="C120" s="16" t="n">
-        <v>2750</v>
+      <c r="C120" s="12" t="n">
+        <v>24697</v>
       </c>
     </row>
     <row r="121" ht="11" customHeight="true" outlineLevel="3">
@@ -2474,7 +2516,7 @@
         <v>120</v>
       </c>
       <c r="C121" s="11" t="n">
-        <v>73</v>
+        <v>55</v>
       </c>
     </row>
     <row r="122" ht="11" customHeight="true" outlineLevel="3">
@@ -2482,7 +2524,7 @@
         <v>121</v>
       </c>
       <c r="C122" s="11" t="n">
-        <v>86</v>
+        <v>68</v>
       </c>
     </row>
     <row r="123" ht="11" customHeight="true" outlineLevel="3">
@@ -2490,7 +2532,7 @@
         <v>122</v>
       </c>
       <c r="C123" s="11" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" ht="11" customHeight="true" outlineLevel="3">
@@ -2498,39 +2540,39 @@
         <v>123</v>
       </c>
       <c r="C124" s="11" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
     </row>
     <row r="125" ht="11" customHeight="true" outlineLevel="3">
       <c r="B125" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="C125" s="11" t="n">
-        <v>150</v>
+      <c r="C125" s="16" t="n">
+        <v>6225</v>
       </c>
     </row>
     <row r="126" ht="11" customHeight="true" outlineLevel="3">
       <c r="B126" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="C126" s="11" t="n">
-        <v>63</v>
+      <c r="C126" s="16" t="n">
+        <v>8219</v>
       </c>
     </row>
     <row r="127" ht="11" customHeight="true" outlineLevel="3">
       <c r="B127" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C127" s="11" t="n">
-        <v>82</v>
+      <c r="C127" s="16" t="n">
+        <v>1700</v>
       </c>
     </row>
     <row r="128" ht="11" customHeight="true" outlineLevel="3">
       <c r="B128" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="C128" s="11" t="n">
-        <v>170</v>
+      <c r="C128" s="16" t="n">
+        <v>1550</v>
       </c>
     </row>
     <row r="129" ht="11" customHeight="true" outlineLevel="3">
@@ -2538,15 +2580,15 @@
         <v>128</v>
       </c>
       <c r="C129" s="11" t="n">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="130" ht="22" customHeight="true" outlineLevel="3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="130" ht="11" customHeight="true" outlineLevel="3">
       <c r="B130" s="15" t="s">
         <v>129</v>
       </c>
       <c r="C130" s="11" t="n">
-        <v>121</v>
+        <v>51</v>
       </c>
     </row>
     <row r="131" ht="11" customHeight="true" outlineLevel="3">
@@ -2554,7 +2596,7 @@
         <v>130</v>
       </c>
       <c r="C131" s="11" t="n">
-        <v>199</v>
+        <v>69</v>
       </c>
     </row>
     <row r="132" ht="11" customHeight="true" outlineLevel="3">
@@ -2562,7 +2604,7 @@
         <v>131</v>
       </c>
       <c r="C132" s="11" t="n">
-        <v>273</v>
+        <v>74</v>
       </c>
     </row>
     <row r="133" ht="11" customHeight="true" outlineLevel="3">
@@ -2570,7 +2612,7 @@
         <v>132</v>
       </c>
       <c r="C133" s="11" t="n">
-        <v>40</v>
+        <v>124</v>
       </c>
     </row>
     <row r="134" ht="11" customHeight="true" outlineLevel="3">
@@ -2578,15 +2620,15 @@
         <v>133</v>
       </c>
       <c r="C134" s="11" t="n">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="135" ht="11" customHeight="true" outlineLevel="3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="135" ht="22" customHeight="true" outlineLevel="3">
       <c r="B135" s="15" t="s">
         <v>134</v>
       </c>
       <c r="C135" s="11" t="n">
-        <v>657</v>
+        <v>64</v>
       </c>
     </row>
     <row r="136" ht="11" customHeight="true" outlineLevel="3">
@@ -2594,7 +2636,7 @@
         <v>135</v>
       </c>
       <c r="C136" s="11" t="n">
-        <v>51</v>
+        <v>268</v>
       </c>
     </row>
     <row r="137" ht="11" customHeight="true" outlineLevel="3">
@@ -2602,7 +2644,7 @@
         <v>136</v>
       </c>
       <c r="C137" s="11" t="n">
-        <v>111</v>
+        <v>40</v>
       </c>
     </row>
     <row r="138" ht="11" customHeight="true" outlineLevel="3">
@@ -2610,7 +2652,7 @@
         <v>137</v>
       </c>
       <c r="C138" s="11" t="n">
-        <v>10</v>
+        <v>768</v>
       </c>
     </row>
     <row r="139" ht="11" customHeight="true" outlineLevel="3">
@@ -2618,7 +2660,7 @@
         <v>138</v>
       </c>
       <c r="C139" s="11" t="n">
-        <v>17</v>
+        <v>77</v>
       </c>
     </row>
     <row r="140" ht="11" customHeight="true" outlineLevel="3">
@@ -2626,7 +2668,7 @@
         <v>139</v>
       </c>
       <c r="C140" s="11" t="n">
-        <v>4</v>
+        <v>766</v>
       </c>
     </row>
     <row r="141" ht="11" customHeight="true" outlineLevel="3">
@@ -2634,7 +2676,7 @@
         <v>140</v>
       </c>
       <c r="C141" s="11" t="n">
-        <v>319</v>
+        <v>377</v>
       </c>
     </row>
     <row r="142" ht="11" customHeight="true" outlineLevel="3">
@@ -2642,7 +2684,7 @@
         <v>141</v>
       </c>
       <c r="C142" s="11" t="n">
-        <v>478</v>
+        <v>39</v>
       </c>
     </row>
     <row r="143" ht="11" customHeight="true" outlineLevel="3">
@@ -2650,15 +2692,15 @@
         <v>142</v>
       </c>
       <c r="C143" s="11" t="n">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="144" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B144" s="14" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="144" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B144" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C144" s="12" t="n">
-        <v>18018</v>
+      <c r="C144" s="11" t="n">
+        <v>89</v>
       </c>
     </row>
     <row r="145" ht="11" customHeight="true" outlineLevel="3">
@@ -2666,7 +2708,7 @@
         <v>144</v>
       </c>
       <c r="C145" s="11" t="n">
-        <v>28</v>
+        <v>638</v>
       </c>
     </row>
     <row r="146" ht="11" customHeight="true" outlineLevel="3">
@@ -2674,7 +2716,7 @@
         <v>145</v>
       </c>
       <c r="C146" s="11" t="n">
-        <v>77</v>
+        <v>248</v>
       </c>
     </row>
     <row r="147" ht="11" customHeight="true" outlineLevel="3">
@@ -2682,7 +2724,7 @@
         <v>146</v>
       </c>
       <c r="C147" s="11" t="n">
-        <v>60</v>
+        <v>766</v>
       </c>
     </row>
     <row r="148" ht="11" customHeight="true" outlineLevel="3">
@@ -2690,7 +2732,7 @@
         <v>147</v>
       </c>
       <c r="C148" s="11" t="n">
-        <v>68</v>
+        <v>248</v>
       </c>
     </row>
     <row r="149" ht="11" customHeight="true" outlineLevel="3">
@@ -2698,7 +2740,7 @@
         <v>148</v>
       </c>
       <c r="C149" s="11" t="n">
-        <v>83</v>
+        <v>768</v>
       </c>
     </row>
     <row r="150" ht="11" customHeight="true" outlineLevel="3">
@@ -2706,7 +2748,7 @@
         <v>149</v>
       </c>
       <c r="C150" s="11" t="n">
-        <v>58</v>
+        <v>192</v>
       </c>
     </row>
     <row r="151" ht="11" customHeight="true" outlineLevel="3">
@@ -2714,15 +2756,15 @@
         <v>150</v>
       </c>
       <c r="C151" s="11" t="n">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="152" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B152" s="15" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="152" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B152" s="14" t="s">
         <v>151</v>
       </c>
-      <c r="C152" s="11" t="n">
-        <v>5</v>
+      <c r="C152" s="12" t="n">
+        <v>13956</v>
       </c>
     </row>
     <row r="153" ht="11" customHeight="true" outlineLevel="3">
@@ -2738,7 +2780,7 @@
         <v>153</v>
       </c>
       <c r="C154" s="11" t="n">
-        <v>476</v>
+        <v>35</v>
       </c>
     </row>
     <row r="155" ht="11" customHeight="true" outlineLevel="3">
@@ -2746,7 +2788,7 @@
         <v>154</v>
       </c>
       <c r="C155" s="11" t="n">
-        <v>165</v>
+        <v>55</v>
       </c>
     </row>
     <row r="156" ht="11" customHeight="true" outlineLevel="3">
@@ -2754,7 +2796,7 @@
         <v>155</v>
       </c>
       <c r="C156" s="11" t="n">
-        <v>255</v>
+        <v>21</v>
       </c>
     </row>
     <row r="157" ht="11" customHeight="true" outlineLevel="3">
@@ -2762,7 +2804,7 @@
         <v>156</v>
       </c>
       <c r="C157" s="11" t="n">
-        <v>75</v>
+        <v>43</v>
       </c>
     </row>
     <row r="158" ht="11" customHeight="true" outlineLevel="3">
@@ -2770,7 +2812,7 @@
         <v>157</v>
       </c>
       <c r="C158" s="11" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="159" ht="11" customHeight="true" outlineLevel="3">
@@ -2778,7 +2820,7 @@
         <v>158</v>
       </c>
       <c r="C159" s="11" t="n">
-        <v>339</v>
+        <v>38</v>
       </c>
     </row>
     <row r="160" ht="11" customHeight="true" outlineLevel="3">
@@ -2786,7 +2828,7 @@
         <v>159</v>
       </c>
       <c r="C160" s="11" t="n">
-        <v>218</v>
+        <v>37</v>
       </c>
     </row>
     <row r="161" ht="11" customHeight="true" outlineLevel="3">
@@ -2794,7 +2836,7 @@
         <v>160</v>
       </c>
       <c r="C161" s="11" t="n">
-        <v>132</v>
+        <v>56</v>
       </c>
     </row>
     <row r="162" ht="11" customHeight="true" outlineLevel="3">
@@ -2802,7 +2844,7 @@
         <v>161</v>
       </c>
       <c r="C162" s="11" t="n">
-        <v>362</v>
+        <v>14</v>
       </c>
     </row>
     <row r="163" ht="11" customHeight="true" outlineLevel="3">
@@ -2810,7 +2852,7 @@
         <v>162</v>
       </c>
       <c r="C163" s="11" t="n">
-        <v>107</v>
+        <v>51</v>
       </c>
     </row>
     <row r="164" ht="11" customHeight="true" outlineLevel="3">
@@ -2818,7 +2860,7 @@
         <v>163</v>
       </c>
       <c r="C164" s="11" t="n">
-        <v>183</v>
+        <v>422</v>
       </c>
     </row>
     <row r="165" ht="11" customHeight="true" outlineLevel="3">
@@ -2826,7 +2868,7 @@
         <v>164</v>
       </c>
       <c r="C165" s="11" t="n">
-        <v>239</v>
+        <v>138</v>
       </c>
     </row>
     <row r="166" ht="11" customHeight="true" outlineLevel="3">
@@ -2834,7 +2876,7 @@
         <v>165</v>
       </c>
       <c r="C166" s="11" t="n">
-        <v>368</v>
+        <v>255</v>
       </c>
     </row>
     <row r="167" ht="11" customHeight="true" outlineLevel="3">
@@ -2842,7 +2884,7 @@
         <v>166</v>
       </c>
       <c r="C167" s="11" t="n">
-        <v>244</v>
+        <v>59</v>
       </c>
     </row>
     <row r="168" ht="11" customHeight="true" outlineLevel="3">
@@ -2850,7 +2892,7 @@
         <v>167</v>
       </c>
       <c r="C168" s="11" t="n">
-        <v>66</v>
+        <v>184</v>
       </c>
     </row>
     <row r="169" ht="11" customHeight="true" outlineLevel="3">
@@ -2858,7 +2900,7 @@
         <v>168</v>
       </c>
       <c r="C169" s="11" t="n">
-        <v>127</v>
+        <v>100</v>
       </c>
     </row>
     <row r="170" ht="11" customHeight="true" outlineLevel="3">
@@ -2866,7 +2908,7 @@
         <v>169</v>
       </c>
       <c r="C170" s="11" t="n">
-        <v>502</v>
+        <v>218</v>
       </c>
     </row>
     <row r="171" ht="11" customHeight="true" outlineLevel="3">
@@ -2874,7 +2916,7 @@
         <v>170</v>
       </c>
       <c r="C171" s="11" t="n">
-        <v>42</v>
+        <v>93</v>
       </c>
     </row>
     <row r="172" ht="11" customHeight="true" outlineLevel="3">
@@ -2882,7 +2924,7 @@
         <v>171</v>
       </c>
       <c r="C172" s="11" t="n">
-        <v>18</v>
+        <v>362</v>
       </c>
     </row>
     <row r="173" ht="11" customHeight="true" outlineLevel="3">
@@ -2890,7 +2932,7 @@
         <v>172</v>
       </c>
       <c r="C173" s="11" t="n">
-        <v>165</v>
+        <v>90</v>
       </c>
     </row>
     <row r="174" ht="11" customHeight="true" outlineLevel="3">
@@ -2898,7 +2940,7 @@
         <v>173</v>
       </c>
       <c r="C174" s="11" t="n">
-        <v>128</v>
+        <v>183</v>
       </c>
     </row>
     <row r="175" ht="11" customHeight="true" outlineLevel="3">
@@ -2906,15 +2948,15 @@
         <v>174</v>
       </c>
       <c r="C175" s="11" t="n">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="176" ht="22" customHeight="true" outlineLevel="3">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="176" ht="11" customHeight="true" outlineLevel="3">
       <c r="B176" s="15" t="s">
         <v>175</v>
       </c>
       <c r="C176" s="11" t="n">
-        <v>44</v>
+        <v>368</v>
       </c>
     </row>
     <row r="177" ht="11" customHeight="true" outlineLevel="3">
@@ -2922,7 +2964,7 @@
         <v>176</v>
       </c>
       <c r="C177" s="11" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="178" ht="11" customHeight="true" outlineLevel="3">
@@ -2930,7 +2972,7 @@
         <v>177</v>
       </c>
       <c r="C178" s="11" t="n">
-        <v>333</v>
+        <v>127</v>
       </c>
     </row>
     <row r="179" ht="11" customHeight="true" outlineLevel="3">
@@ -2938,7 +2980,7 @@
         <v>178</v>
       </c>
       <c r="C179" s="11" t="n">
-        <v>17</v>
+        <v>53</v>
       </c>
     </row>
     <row r="180" ht="11" customHeight="true" outlineLevel="3">
@@ -2946,23 +2988,23 @@
         <v>179</v>
       </c>
       <c r="C180" s="11" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="181" ht="22" customHeight="true" outlineLevel="3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="181" ht="11" customHeight="true" outlineLevel="3">
       <c r="B181" s="15" t="s">
         <v>180</v>
       </c>
       <c r="C181" s="11" t="n">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="182" ht="22" customHeight="true" outlineLevel="3">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="182" ht="11" customHeight="true" outlineLevel="3">
       <c r="B182" s="15" t="s">
         <v>181</v>
       </c>
       <c r="C182" s="11" t="n">
-        <v>138</v>
+        <v>408</v>
       </c>
     </row>
     <row r="183" ht="11" customHeight="true" outlineLevel="3">
@@ -2970,7 +3012,7 @@
         <v>182</v>
       </c>
       <c r="C183" s="11" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
     </row>
     <row r="184" ht="11" customHeight="true" outlineLevel="3">
@@ -2978,15 +3020,15 @@
         <v>183</v>
       </c>
       <c r="C184" s="11" t="n">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="185" ht="22" customHeight="true" outlineLevel="3">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="185" ht="11" customHeight="true" outlineLevel="3">
       <c r="B185" s="15" t="s">
         <v>184</v>
       </c>
       <c r="C185" s="11" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="186" ht="11" customHeight="true" outlineLevel="3">
@@ -2994,7 +3036,7 @@
         <v>185</v>
       </c>
       <c r="C186" s="11" t="n">
-        <v>51</v>
+        <v>14</v>
       </c>
     </row>
     <row r="187" ht="22" customHeight="true" outlineLevel="3">
@@ -3002,15 +3044,15 @@
         <v>186</v>
       </c>
       <c r="C187" s="11" t="n">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="188" ht="11" customHeight="true" outlineLevel="3">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="188" ht="22" customHeight="true" outlineLevel="3">
       <c r="B188" s="15" t="s">
         <v>187</v>
       </c>
       <c r="C188" s="11" t="n">
-        <v>112</v>
+        <v>127</v>
       </c>
     </row>
     <row r="189" ht="11" customHeight="true" outlineLevel="3">
@@ -3018,7 +3060,7 @@
         <v>188</v>
       </c>
       <c r="C189" s="11" t="n">
-        <v>427</v>
+        <v>25</v>
       </c>
     </row>
     <row r="190" ht="11" customHeight="true" outlineLevel="3">
@@ -3026,15 +3068,15 @@
         <v>189</v>
       </c>
       <c r="C190" s="11" t="n">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="191" ht="11" customHeight="true" outlineLevel="3">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="191" ht="22" customHeight="true" outlineLevel="3">
       <c r="B191" s="15" t="s">
         <v>190</v>
       </c>
       <c r="C191" s="11" t="n">
-        <v>169</v>
+        <v>9</v>
       </c>
     </row>
     <row r="192" ht="11" customHeight="true" outlineLevel="3">
@@ -3042,15 +3084,15 @@
         <v>191</v>
       </c>
       <c r="C192" s="11" t="n">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="193" ht="11" customHeight="true" outlineLevel="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="193" ht="22" customHeight="true" outlineLevel="3">
       <c r="B193" s="15" t="s">
         <v>192</v>
       </c>
       <c r="C193" s="11" t="n">
-        <v>179</v>
+        <v>135</v>
       </c>
     </row>
     <row r="194" ht="11" customHeight="true" outlineLevel="3">
@@ -3058,7 +3100,7 @@
         <v>193</v>
       </c>
       <c r="C194" s="11" t="n">
-        <v>314</v>
+        <v>97</v>
       </c>
     </row>
     <row r="195" ht="11" customHeight="true" outlineLevel="3">
@@ -3066,7 +3108,7 @@
         <v>194</v>
       </c>
       <c r="C195" s="11" t="n">
-        <v>100</v>
+        <v>427</v>
       </c>
     </row>
     <row r="196" ht="11" customHeight="true" outlineLevel="3">
@@ -3074,7 +3116,7 @@
         <v>195</v>
       </c>
       <c r="C196" s="11" t="n">
-        <v>225</v>
+        <v>3</v>
       </c>
     </row>
     <row r="197" ht="11" customHeight="true" outlineLevel="3">
@@ -3082,7 +3124,7 @@
         <v>196</v>
       </c>
       <c r="C197" s="11" t="n">
-        <v>91</v>
+        <v>152</v>
       </c>
     </row>
     <row r="198" ht="11" customHeight="true" outlineLevel="3">
@@ -3090,7 +3132,7 @@
         <v>197</v>
       </c>
       <c r="C198" s="11" t="n">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="199" ht="11" customHeight="true" outlineLevel="3">
@@ -3098,15 +3140,15 @@
         <v>198</v>
       </c>
       <c r="C199" s="11" t="n">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="200" ht="22" customHeight="true" outlineLevel="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="200" ht="11" customHeight="true" outlineLevel="3">
       <c r="B200" s="15" t="s">
         <v>199</v>
       </c>
       <c r="C200" s="11" t="n">
-        <v>44</v>
+        <v>314</v>
       </c>
     </row>
     <row r="201" ht="11" customHeight="true" outlineLevel="3">
@@ -3114,7 +3156,7 @@
         <v>200</v>
       </c>
       <c r="C201" s="11" t="n">
-        <v>68</v>
+        <v>244</v>
       </c>
     </row>
     <row r="202" ht="11" customHeight="true" outlineLevel="3">
@@ -3122,7 +3164,7 @@
         <v>201</v>
       </c>
       <c r="C202" s="11" t="n">
-        <v>112</v>
+        <v>225</v>
       </c>
     </row>
     <row r="203" ht="11" customHeight="true" outlineLevel="3">
@@ -3130,7 +3172,7 @@
         <v>202</v>
       </c>
       <c r="C203" s="11" t="n">
-        <v>63</v>
+        <v>173</v>
       </c>
     </row>
     <row r="204" ht="11" customHeight="true" outlineLevel="3">
@@ -3138,7 +3180,7 @@
         <v>203</v>
       </c>
       <c r="C204" s="11" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="205" ht="11" customHeight="true" outlineLevel="3">
@@ -3146,7 +3188,7 @@
         <v>204</v>
       </c>
       <c r="C205" s="11" t="n">
-        <v>199</v>
+        <v>244</v>
       </c>
     </row>
     <row r="206" ht="11" customHeight="true" outlineLevel="3">
@@ -3154,7 +3196,7 @@
         <v>205</v>
       </c>
       <c r="C206" s="11" t="n">
-        <v>92</v>
+        <v>5</v>
       </c>
     </row>
     <row r="207" ht="11" customHeight="true" outlineLevel="3">
@@ -3162,7 +3204,7 @@
         <v>206</v>
       </c>
       <c r="C207" s="11" t="n">
-        <v>418</v>
+        <v>57</v>
       </c>
     </row>
     <row r="208" ht="11" customHeight="true" outlineLevel="3">
@@ -3170,7 +3212,7 @@
         <v>207</v>
       </c>
       <c r="C208" s="11" t="n">
-        <v>384</v>
+        <v>112</v>
       </c>
     </row>
     <row r="209" ht="11" customHeight="true" outlineLevel="3">
@@ -3178,7 +3220,7 @@
         <v>208</v>
       </c>
       <c r="C209" s="11" t="n">
-        <v>13</v>
+        <v>55</v>
       </c>
     </row>
     <row r="210" ht="11" customHeight="true" outlineLevel="3">
@@ -3186,7 +3228,7 @@
         <v>209</v>
       </c>
       <c r="C210" s="11" t="n">
-        <v>211</v>
+        <v>5</v>
       </c>
     </row>
     <row r="211" ht="11" customHeight="true" outlineLevel="3">
@@ -3194,7 +3236,7 @@
         <v>210</v>
       </c>
       <c r="C211" s="11" t="n">
-        <v>131</v>
+        <v>106</v>
       </c>
     </row>
     <row r="212" ht="11" customHeight="true" outlineLevel="3">
@@ -3202,7 +3244,7 @@
         <v>211</v>
       </c>
       <c r="C212" s="11" t="n">
-        <v>271</v>
+        <v>145</v>
       </c>
     </row>
     <row r="213" ht="11" customHeight="true" outlineLevel="3">
@@ -3210,15 +3252,15 @@
         <v>212</v>
       </c>
       <c r="C213" s="11" t="n">
-        <v>154</v>
+        <v>189</v>
       </c>
     </row>
     <row r="214" ht="11" customHeight="true" outlineLevel="3">
       <c r="B214" s="15" t="s">
         <v>213</v>
       </c>
-      <c r="C214" s="16" t="n">
-        <v>1008</v>
+      <c r="C214" s="11" t="n">
+        <v>92</v>
       </c>
     </row>
     <row r="215" ht="11" customHeight="true" outlineLevel="3">
@@ -3226,15 +3268,15 @@
         <v>214</v>
       </c>
       <c r="C215" s="11" t="n">
-        <v>296</v>
+        <v>146</v>
       </c>
     </row>
     <row r="216" ht="11" customHeight="true" outlineLevel="3">
       <c r="B216" s="15" t="s">
         <v>215</v>
       </c>
-      <c r="C216" s="16" t="n">
-        <v>2908</v>
+      <c r="C216" s="11" t="n">
+        <v>384</v>
       </c>
     </row>
     <row r="217" ht="11" customHeight="true" outlineLevel="3">
@@ -3242,7 +3284,7 @@
         <v>216</v>
       </c>
       <c r="C217" s="11" t="n">
-        <v>275</v>
+        <v>131</v>
       </c>
     </row>
     <row r="218" ht="11" customHeight="true" outlineLevel="3">
@@ -3250,7 +3292,7 @@
         <v>217</v>
       </c>
       <c r="C218" s="11" t="n">
-        <v>183</v>
+        <v>131</v>
       </c>
     </row>
     <row r="219" ht="11" customHeight="true" outlineLevel="3">
@@ -3258,7 +3300,7 @@
         <v>218</v>
       </c>
       <c r="C219" s="11" t="n">
-        <v>184</v>
+        <v>34</v>
       </c>
     </row>
     <row r="220" ht="11" customHeight="true" outlineLevel="3">
@@ -3266,7 +3308,7 @@
         <v>219</v>
       </c>
       <c r="C220" s="11" t="n">
-        <v>662</v>
+        <v>152</v>
       </c>
     </row>
     <row r="221" ht="11" customHeight="true" outlineLevel="3">
@@ -3274,7 +3316,7 @@
         <v>220</v>
       </c>
       <c r="C221" s="11" t="n">
-        <v>135</v>
+        <v>154</v>
       </c>
     </row>
     <row r="222" ht="11" customHeight="true" outlineLevel="3">
@@ -3282,15 +3324,15 @@
         <v>221</v>
       </c>
       <c r="C222" s="11" t="n">
-        <v>293</v>
+        <v>76</v>
       </c>
     </row>
     <row r="223" ht="11" customHeight="true" outlineLevel="3">
       <c r="B223" s="15" t="s">
         <v>222</v>
       </c>
-      <c r="C223" s="11" t="n">
-        <v>2</v>
+      <c r="C223" s="16" t="n">
+        <v>2688</v>
       </c>
     </row>
     <row r="224" ht="11" customHeight="true" outlineLevel="3">
@@ -3298,7 +3340,7 @@
         <v>223</v>
       </c>
       <c r="C224" s="11" t="n">
-        <v>195</v>
+        <v>275</v>
       </c>
     </row>
     <row r="225" ht="11" customHeight="true" outlineLevel="3">
@@ -3306,7 +3348,7 @@
         <v>224</v>
       </c>
       <c r="C225" s="11" t="n">
-        <v>111</v>
+        <v>173</v>
       </c>
     </row>
     <row r="226" ht="11" customHeight="true" outlineLevel="3">
@@ -3314,7 +3356,7 @@
         <v>225</v>
       </c>
       <c r="C226" s="11" t="n">
-        <v>263</v>
+        <v>184</v>
       </c>
     </row>
     <row r="227" ht="11" customHeight="true" outlineLevel="3">
@@ -3322,7 +3364,7 @@
         <v>226</v>
       </c>
       <c r="C227" s="11" t="n">
-        <v>31</v>
+        <v>237</v>
       </c>
     </row>
     <row r="228" ht="11" customHeight="true" outlineLevel="3">
@@ -3330,7 +3372,7 @@
         <v>227</v>
       </c>
       <c r="C228" s="11" t="n">
-        <v>253</v>
+        <v>293</v>
       </c>
     </row>
     <row r="229" ht="11" customHeight="true" outlineLevel="3">
@@ -3338,15 +3380,15 @@
         <v>228</v>
       </c>
       <c r="C229" s="11" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="230" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B230" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="230" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B230" s="15" t="s">
         <v>229</v>
       </c>
-      <c r="C230" s="12" t="n">
-        <v>9859</v>
+      <c r="C230" s="11" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="231" ht="11" customHeight="true" outlineLevel="3">
@@ -3354,7 +3396,7 @@
         <v>230</v>
       </c>
       <c r="C231" s="11" t="n">
-        <v>226</v>
+        <v>89</v>
       </c>
     </row>
     <row r="232" ht="11" customHeight="true" outlineLevel="3">
@@ -3362,7 +3404,7 @@
         <v>231</v>
       </c>
       <c r="C232" s="11" t="n">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="233" ht="11" customHeight="true" outlineLevel="3">
@@ -3370,7 +3412,7 @@
         <v>232</v>
       </c>
       <c r="C233" s="11" t="n">
-        <v>222</v>
+        <v>14</v>
       </c>
     </row>
     <row r="234" ht="11" customHeight="true" outlineLevel="3">
@@ -3378,7 +3420,7 @@
         <v>233</v>
       </c>
       <c r="C234" s="11" t="n">
-        <v>234</v>
+        <v>229</v>
       </c>
     </row>
     <row r="235" ht="11" customHeight="true" outlineLevel="3">
@@ -3386,15 +3428,15 @@
         <v>234</v>
       </c>
       <c r="C235" s="11" t="n">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="236" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B236" s="15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="236" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B236" s="14" t="s">
         <v>235</v>
       </c>
-      <c r="C236" s="11" t="n">
-        <v>763</v>
+      <c r="C236" s="12" t="n">
+        <v>5714</v>
       </c>
     </row>
     <row r="237" ht="11" customHeight="true" outlineLevel="3">
@@ -3402,7 +3444,7 @@
         <v>236</v>
       </c>
       <c r="C237" s="11" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="238" ht="11" customHeight="true" outlineLevel="3">
@@ -3410,7 +3452,7 @@
         <v>237</v>
       </c>
       <c r="C238" s="11" t="n">
-        <v>74</v>
+        <v>339</v>
       </c>
     </row>
     <row r="239" ht="11" customHeight="true" outlineLevel="3">
@@ -3418,7 +3460,7 @@
         <v>238</v>
       </c>
       <c r="C239" s="11" t="n">
-        <v>82</v>
+        <v>224</v>
       </c>
     </row>
     <row r="240" ht="11" customHeight="true" outlineLevel="3">
@@ -3426,7 +3468,7 @@
         <v>239</v>
       </c>
       <c r="C240" s="11" t="n">
-        <v>220</v>
+        <v>139</v>
       </c>
     </row>
     <row r="241" ht="11" customHeight="true" outlineLevel="3">
@@ -3434,7 +3476,7 @@
         <v>240</v>
       </c>
       <c r="C241" s="11" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="242" ht="11" customHeight="true" outlineLevel="3">
@@ -3442,7 +3484,7 @@
         <v>241</v>
       </c>
       <c r="C242" s="11" t="n">
-        <v>78</v>
+        <v>473</v>
       </c>
     </row>
     <row r="243" ht="11" customHeight="true" outlineLevel="3">
@@ -3450,7 +3492,7 @@
         <v>242</v>
       </c>
       <c r="C243" s="11" t="n">
-        <v>560</v>
+        <v>30</v>
       </c>
     </row>
     <row r="244" ht="11" customHeight="true" outlineLevel="3">
@@ -3458,7 +3500,7 @@
         <v>243</v>
       </c>
       <c r="C244" s="11" t="n">
-        <v>43</v>
+        <v>74</v>
       </c>
     </row>
     <row r="245" ht="11" customHeight="true" outlineLevel="3">
@@ -3466,7 +3508,7 @@
         <v>244</v>
       </c>
       <c r="C245" s="11" t="n">
-        <v>441</v>
+        <v>39</v>
       </c>
     </row>
     <row r="246" ht="11" customHeight="true" outlineLevel="3">
@@ -3474,7 +3516,7 @@
         <v>245</v>
       </c>
       <c r="C246" s="11" t="n">
-        <v>24</v>
+        <v>78</v>
       </c>
     </row>
     <row r="247" ht="11" customHeight="true" outlineLevel="3">
@@ -3482,7 +3524,7 @@
         <v>246</v>
       </c>
       <c r="C247" s="11" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="248" ht="11" customHeight="true" outlineLevel="3">
@@ -3490,7 +3532,7 @@
         <v>247</v>
       </c>
       <c r="C248" s="11" t="n">
-        <v>165</v>
+        <v>202</v>
       </c>
     </row>
     <row r="249" ht="11" customHeight="true" outlineLevel="3">
@@ -3498,7 +3540,7 @@
         <v>248</v>
       </c>
       <c r="C249" s="11" t="n">
-        <v>57</v>
+        <v>241</v>
       </c>
     </row>
     <row r="250" ht="11" customHeight="true" outlineLevel="3">
@@ -3506,7 +3548,7 @@
         <v>249</v>
       </c>
       <c r="C250" s="11" t="n">
-        <v>499</v>
+        <v>18</v>
       </c>
     </row>
     <row r="251" ht="11" customHeight="true" outlineLevel="3">
@@ -3514,7 +3556,7 @@
         <v>250</v>
       </c>
       <c r="C251" s="11" t="n">
-        <v>8</v>
+        <v>54</v>
       </c>
     </row>
     <row r="252" ht="11" customHeight="true" outlineLevel="3">
@@ -3522,7 +3564,7 @@
         <v>251</v>
       </c>
       <c r="C252" s="11" t="n">
-        <v>433</v>
+        <v>54</v>
       </c>
     </row>
     <row r="253" ht="11" customHeight="true" outlineLevel="3">
@@ -3530,7 +3572,7 @@
         <v>252</v>
       </c>
       <c r="C253" s="11" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="254" ht="11" customHeight="true" outlineLevel="3">
@@ -3538,7 +3580,7 @@
         <v>253</v>
       </c>
       <c r="C254" s="11" t="n">
-        <v>631</v>
+        <v>430</v>
       </c>
     </row>
     <row r="255" ht="11" customHeight="true" outlineLevel="3">
@@ -3546,7 +3588,7 @@
         <v>254</v>
       </c>
       <c r="C255" s="11" t="n">
-        <v>119</v>
+        <v>216</v>
       </c>
     </row>
     <row r="256" ht="11" customHeight="true" outlineLevel="3">
@@ -3554,7 +3596,7 @@
         <v>255</v>
       </c>
       <c r="C256" s="11" t="n">
-        <v>212</v>
+        <v>119</v>
       </c>
     </row>
     <row r="257" ht="11" customHeight="true" outlineLevel="3">
@@ -3562,7 +3604,7 @@
         <v>256</v>
       </c>
       <c r="C257" s="11" t="n">
-        <v>414</v>
+        <v>408</v>
       </c>
     </row>
     <row r="258" ht="11" customHeight="true" outlineLevel="3">
@@ -3570,7 +3612,7 @@
         <v>257</v>
       </c>
       <c r="C258" s="11" t="n">
-        <v>258</v>
+        <v>225</v>
       </c>
     </row>
     <row r="259" ht="11" customHeight="true" outlineLevel="3">
@@ -3578,7 +3620,7 @@
         <v>258</v>
       </c>
       <c r="C259" s="11" t="n">
-        <v>414</v>
+        <v>253</v>
       </c>
     </row>
     <row r="260" ht="11" customHeight="true" outlineLevel="3">
@@ -3586,7 +3628,7 @@
         <v>259</v>
       </c>
       <c r="C260" s="11" t="n">
-        <v>295</v>
+        <v>599</v>
       </c>
     </row>
     <row r="261" ht="11" customHeight="true" outlineLevel="3">
@@ -3594,7 +3636,7 @@
         <v>260</v>
       </c>
       <c r="C261" s="11" t="n">
-        <v>624</v>
+        <v>194</v>
       </c>
     </row>
     <row r="262" ht="11" customHeight="true" outlineLevel="3">
@@ -3602,7 +3644,7 @@
         <v>261</v>
       </c>
       <c r="C262" s="11" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="263" ht="11" customHeight="true" outlineLevel="3">
@@ -3610,15 +3652,15 @@
         <v>262</v>
       </c>
       <c r="C263" s="11" t="n">
-        <v>230</v>
+        <v>24</v>
       </c>
     </row>
     <row r="264" ht="11" customHeight="true" outlineLevel="3">
       <c r="B264" s="15" t="s">
         <v>263</v>
       </c>
-      <c r="C264" s="16" t="n">
-        <v>1792</v>
+      <c r="C264" s="11" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="265" ht="11" customHeight="true" outlineLevel="3">
@@ -3626,15 +3668,15 @@
         <v>264</v>
       </c>
       <c r="C265" s="11" t="n">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="266" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B266" s="14" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="266" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B266" s="15" t="s">
         <v>265</v>
       </c>
-      <c r="C266" s="17" t="n">
-        <v>678</v>
+      <c r="C266" s="11" t="n">
+        <v>383</v>
       </c>
     </row>
     <row r="267" ht="11" customHeight="true" outlineLevel="3">
@@ -3642,7 +3684,7 @@
         <v>266</v>
       </c>
       <c r="C267" s="11" t="n">
-        <v>62</v>
+        <v>176</v>
       </c>
     </row>
     <row r="268" ht="11" customHeight="true" outlineLevel="3">
@@ -3650,7 +3692,7 @@
         <v>267</v>
       </c>
       <c r="C268" s="11" t="n">
-        <v>1</v>
+        <v>335</v>
       </c>
     </row>
     <row r="269" ht="11" customHeight="true" outlineLevel="3">
@@ -3658,7 +3700,7 @@
         <v>268</v>
       </c>
       <c r="C269" s="11" t="n">
-        <v>25</v>
+        <v>71</v>
       </c>
     </row>
     <row r="270" ht="11" customHeight="true" outlineLevel="3">
@@ -3666,15 +3708,15 @@
         <v>269</v>
       </c>
       <c r="C270" s="11" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="271" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B271" s="15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="271" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B271" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="C271" s="11" t="n">
-        <v>25</v>
+      <c r="C271" s="17" t="n">
+        <v>531</v>
       </c>
     </row>
     <row r="272" ht="11" customHeight="true" outlineLevel="3">
@@ -3682,7 +3724,7 @@
         <v>271</v>
       </c>
       <c r="C272" s="11" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
     </row>
     <row r="273" ht="11" customHeight="true" outlineLevel="3">
@@ -3690,7 +3732,7 @@
         <v>272</v>
       </c>
       <c r="C273" s="11" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="274" ht="11" customHeight="true" outlineLevel="3">
@@ -3698,7 +3740,7 @@
         <v>273</v>
       </c>
       <c r="C274" s="11" t="n">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
     <row r="275" ht="11" customHeight="true" outlineLevel="3">
@@ -3706,7 +3748,7 @@
         <v>274</v>
       </c>
       <c r="C275" s="11" t="n">
-        <v>53</v>
+        <v>5</v>
       </c>
     </row>
     <row r="276" ht="11" customHeight="true" outlineLevel="3">
@@ -3714,7 +3756,7 @@
         <v>275</v>
       </c>
       <c r="C276" s="11" t="n">
-        <v>248</v>
+        <v>25</v>
       </c>
     </row>
     <row r="277" ht="11" customHeight="true" outlineLevel="3">
@@ -3722,7 +3764,7 @@
         <v>276</v>
       </c>
       <c r="C277" s="11" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
     </row>
     <row r="278" ht="11" customHeight="true" outlineLevel="3">
@@ -3738,7 +3780,7 @@
         <v>278</v>
       </c>
       <c r="C279" s="11" t="n">
-        <v>69</v>
+        <v>10</v>
       </c>
     </row>
     <row r="280" ht="11" customHeight="true" outlineLevel="3">
@@ -3746,7 +3788,7 @@
         <v>279</v>
       </c>
       <c r="C280" s="11" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
     </row>
     <row r="281" ht="11" customHeight="true" outlineLevel="3">
@@ -3754,15 +3796,15 @@
         <v>280</v>
       </c>
       <c r="C281" s="11" t="n">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="282" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B282" s="14" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="282" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B282" s="15" t="s">
         <v>281</v>
       </c>
-      <c r="C282" s="12" t="n">
-        <v>9574</v>
+      <c r="C282" s="11" t="n">
+        <v>226</v>
       </c>
     </row>
     <row r="283" ht="11" customHeight="true" outlineLevel="3">
@@ -3770,7 +3812,7 @@
         <v>282</v>
       </c>
       <c r="C283" s="11" t="n">
-        <v>474</v>
+        <v>32</v>
       </c>
     </row>
     <row r="284" ht="11" customHeight="true" outlineLevel="3">
@@ -3778,7 +3820,7 @@
         <v>283</v>
       </c>
       <c r="C284" s="11" t="n">
-        <v>163</v>
+        <v>46</v>
       </c>
     </row>
     <row r="285" ht="11" customHeight="true" outlineLevel="3">
@@ -3786,7 +3828,7 @@
         <v>284</v>
       </c>
       <c r="C285" s="11" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="286" ht="11" customHeight="true" outlineLevel="3">
@@ -3794,7 +3836,7 @@
         <v>285</v>
       </c>
       <c r="C286" s="11" t="n">
-        <v>129</v>
+        <v>12</v>
       </c>
     </row>
     <row r="287" ht="11" customHeight="true" outlineLevel="3">
@@ -3802,15 +3844,15 @@
         <v>286</v>
       </c>
       <c r="C287" s="11" t="n">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="288" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B288" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="288" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B288" s="14" t="s">
         <v>287</v>
       </c>
-      <c r="C288" s="11" t="n">
-        <v>184</v>
+      <c r="C288" s="12" t="n">
+        <v>9087</v>
       </c>
     </row>
     <row r="289" ht="11" customHeight="true" outlineLevel="3">
@@ -3818,7 +3860,7 @@
         <v>288</v>
       </c>
       <c r="C289" s="11" t="n">
-        <v>26</v>
+        <v>428</v>
       </c>
     </row>
     <row r="290" ht="11" customHeight="true" outlineLevel="3">
@@ -3826,15 +3868,15 @@
         <v>289</v>
       </c>
       <c r="C290" s="11" t="n">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="291" ht="22" customHeight="true" outlineLevel="3">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="291" ht="11" customHeight="true" outlineLevel="3">
       <c r="B291" s="15" t="s">
         <v>290</v>
       </c>
       <c r="C291" s="11" t="n">
-        <v>56</v>
+        <v>141</v>
       </c>
     </row>
     <row r="292" ht="11" customHeight="true" outlineLevel="3">
@@ -3842,7 +3884,7 @@
         <v>291</v>
       </c>
       <c r="C292" s="11" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
     </row>
     <row r="293" ht="11" customHeight="true" outlineLevel="3">
@@ -3850,7 +3892,7 @@
         <v>292</v>
       </c>
       <c r="C293" s="11" t="n">
-        <v>116</v>
+        <v>110</v>
       </c>
     </row>
     <row r="294" ht="11" customHeight="true" outlineLevel="3">
@@ -3858,23 +3900,23 @@
         <v>293</v>
       </c>
       <c r="C294" s="11" t="n">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="295" ht="22" customHeight="true" outlineLevel="3">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="295" ht="11" customHeight="true" outlineLevel="3">
       <c r="B295" s="15" t="s">
         <v>294</v>
       </c>
       <c r="C295" s="11" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="296" ht="22" customHeight="true" outlineLevel="3">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="296" ht="11" customHeight="true" outlineLevel="3">
       <c r="B296" s="15" t="s">
         <v>295</v>
       </c>
       <c r="C296" s="11" t="n">
-        <v>23</v>
+        <v>151</v>
       </c>
     </row>
     <row r="297" ht="22" customHeight="true" outlineLevel="3">
@@ -3882,31 +3924,31 @@
         <v>296</v>
       </c>
       <c r="C297" s="11" t="n">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="298" ht="22" customHeight="true" outlineLevel="3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="298" ht="11" customHeight="true" outlineLevel="3">
       <c r="B298" s="15" t="s">
         <v>297</v>
       </c>
       <c r="C298" s="11" t="n">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="299" ht="22" customHeight="true" outlineLevel="3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="299" ht="11" customHeight="true" outlineLevel="3">
       <c r="B299" s="15" t="s">
         <v>298</v>
       </c>
       <c r="C299" s="11" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="300" ht="22" customHeight="true" outlineLevel="3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="300" ht="11" customHeight="true" outlineLevel="3">
       <c r="B300" s="15" t="s">
         <v>299</v>
       </c>
       <c r="C300" s="11" t="n">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="301" ht="11" customHeight="true" outlineLevel="3">
@@ -3914,7 +3956,7 @@
         <v>300</v>
       </c>
       <c r="C301" s="11" t="n">
-        <v>71</v>
+        <v>26</v>
       </c>
     </row>
     <row r="302" ht="11" customHeight="true" outlineLevel="3">
@@ -3922,31 +3964,31 @@
         <v>301</v>
       </c>
       <c r="C302" s="11" t="n">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="303" ht="11" customHeight="true" outlineLevel="3">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="303" ht="22" customHeight="true" outlineLevel="3">
       <c r="B303" s="15" t="s">
         <v>302</v>
       </c>
       <c r="C303" s="11" t="n">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="304" ht="11" customHeight="true" outlineLevel="3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="304" ht="22" customHeight="true" outlineLevel="3">
       <c r="B304" s="15" t="s">
         <v>303</v>
       </c>
       <c r="C304" s="11" t="n">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="305" ht="11" customHeight="true" outlineLevel="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="305" ht="22" customHeight="true" outlineLevel="3">
       <c r="B305" s="15" t="s">
         <v>304</v>
       </c>
       <c r="C305" s="11" t="n">
-        <v>660</v>
+        <v>9</v>
       </c>
     </row>
     <row r="306" ht="22" customHeight="true" outlineLevel="3">
@@ -3954,23 +3996,23 @@
         <v>305</v>
       </c>
       <c r="C306" s="11" t="n">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="307" ht="11" customHeight="true" outlineLevel="3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="307" ht="22" customHeight="true" outlineLevel="3">
       <c r="B307" s="15" t="s">
         <v>306</v>
       </c>
-      <c r="C307" s="16" t="n">
-        <v>1897</v>
-      </c>
-    </row>
-    <row r="308" ht="11" customHeight="true" outlineLevel="3">
+      <c r="C307" s="11" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="308" ht="22" customHeight="true" outlineLevel="3">
       <c r="B308" s="15" t="s">
         <v>307</v>
       </c>
       <c r="C308" s="11" t="n">
-        <v>55</v>
+        <v>27</v>
       </c>
     </row>
     <row r="309" ht="11" customHeight="true" outlineLevel="3">
@@ -3978,7 +4020,7 @@
         <v>308</v>
       </c>
       <c r="C309" s="11" t="n">
-        <v>918</v>
+        <v>26</v>
       </c>
     </row>
     <row r="310" ht="11" customHeight="true" outlineLevel="3">
@@ -3986,7 +4028,7 @@
         <v>309</v>
       </c>
       <c r="C310" s="11" t="n">
-        <v>123</v>
+        <v>30</v>
       </c>
     </row>
     <row r="311" ht="11" customHeight="true" outlineLevel="3">
@@ -3994,7 +4036,7 @@
         <v>310</v>
       </c>
       <c r="C311" s="11" t="n">
-        <v>299</v>
+        <v>71</v>
       </c>
     </row>
     <row r="312" ht="11" customHeight="true" outlineLevel="3">
@@ -4002,7 +4044,7 @@
         <v>311</v>
       </c>
       <c r="C312" s="11" t="n">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="313" ht="11" customHeight="true" outlineLevel="3">
@@ -4010,23 +4052,23 @@
         <v>312</v>
       </c>
       <c r="C313" s="11" t="n">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="314" ht="11" customHeight="true" outlineLevel="3">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="314" ht="22" customHeight="true" outlineLevel="3">
       <c r="B314" s="15" t="s">
         <v>313</v>
       </c>
-      <c r="C314" s="16" t="n">
-        <v>2002</v>
+      <c r="C314" s="11" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="315" ht="11" customHeight="true" outlineLevel="3">
       <c r="B315" s="15" t="s">
         <v>314</v>
       </c>
-      <c r="C315" s="11" t="n">
-        <v>105</v>
+      <c r="C315" s="16" t="n">
+        <v>1479</v>
       </c>
     </row>
     <row r="316" ht="11" customHeight="true" outlineLevel="3">
@@ -4034,15 +4076,15 @@
         <v>315</v>
       </c>
       <c r="C316" s="11" t="n">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="317" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B317" s="14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="317" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B317" s="15" t="s">
         <v>316</v>
       </c>
-      <c r="C317" s="12" t="n">
-        <v>10345</v>
+      <c r="C317" s="11" t="n">
+        <v>588</v>
       </c>
     </row>
     <row r="318" ht="11" customHeight="true" outlineLevel="3">
@@ -4050,7 +4092,7 @@
         <v>317</v>
       </c>
       <c r="C318" s="11" t="n">
-        <v>646</v>
+        <v>399</v>
       </c>
     </row>
     <row r="319" ht="11" customHeight="true" outlineLevel="3">
@@ -4058,15 +4100,15 @@
         <v>318</v>
       </c>
       <c r="C319" s="11" t="n">
-        <v>978</v>
-      </c>
-    </row>
-    <row r="320" ht="22" customHeight="true" outlineLevel="3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="320" ht="11" customHeight="true" outlineLevel="3">
       <c r="B320" s="15" t="s">
         <v>319</v>
       </c>
       <c r="C320" s="11" t="n">
-        <v>9</v>
+        <v>282</v>
       </c>
     </row>
     <row r="321" ht="11" customHeight="true" outlineLevel="3">
@@ -4074,7 +4116,7 @@
         <v>320</v>
       </c>
       <c r="C321" s="11" t="n">
-        <v>748</v>
+        <v>118</v>
       </c>
     </row>
     <row r="322" ht="11" customHeight="true" outlineLevel="3">
@@ -4082,23 +4124,23 @@
         <v>321</v>
       </c>
       <c r="C322" s="11" t="n">
-        <v>266</v>
+        <v>236</v>
       </c>
     </row>
     <row r="323" ht="11" customHeight="true" outlineLevel="3">
       <c r="B323" s="15" t="s">
         <v>322</v>
       </c>
-      <c r="C323" s="11" t="n">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="324" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B324" s="15" t="s">
+      <c r="C323" s="16" t="n">
+        <v>3057</v>
+      </c>
+    </row>
+    <row r="324" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B324" s="14" t="s">
         <v>323</v>
       </c>
-      <c r="C324" s="11" t="n">
-        <v>982</v>
+      <c r="C324" s="12" t="n">
+        <v>6802</v>
       </c>
     </row>
     <row r="325" ht="11" customHeight="true" outlineLevel="3">
@@ -4106,7 +4148,7 @@
         <v>324</v>
       </c>
       <c r="C325" s="11" t="n">
-        <v>57</v>
+        <v>398</v>
       </c>
     </row>
     <row r="326" ht="11" customHeight="true" outlineLevel="3">
@@ -4114,23 +4156,23 @@
         <v>325</v>
       </c>
       <c r="C326" s="11" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="327" ht="11" customHeight="true" outlineLevel="3">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="327" ht="22" customHeight="true" outlineLevel="3">
       <c r="B327" s="15" t="s">
         <v>326</v>
       </c>
       <c r="C327" s="11" t="n">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="328" ht="11" customHeight="true" outlineLevel="3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="328" ht="22" customHeight="true" outlineLevel="3">
       <c r="B328" s="15" t="s">
         <v>327</v>
       </c>
       <c r="C328" s="11" t="n">
-        <v>96</v>
+        <v>18</v>
       </c>
     </row>
     <row r="329" ht="11" customHeight="true" outlineLevel="3">
@@ -4138,7 +4180,7 @@
         <v>328</v>
       </c>
       <c r="C329" s="11" t="n">
-        <v>105</v>
+        <v>301</v>
       </c>
     </row>
     <row r="330" ht="11" customHeight="true" outlineLevel="3">
@@ -4146,7 +4188,7 @@
         <v>329</v>
       </c>
       <c r="C330" s="11" t="n">
-        <v>189</v>
+        <v>4</v>
       </c>
     </row>
     <row r="331" ht="11" customHeight="true" outlineLevel="3">
@@ -4154,7 +4196,7 @@
         <v>330</v>
       </c>
       <c r="C331" s="11" t="n">
-        <v>597</v>
+        <v>154</v>
       </c>
     </row>
     <row r="332" ht="11" customHeight="true" outlineLevel="3">
@@ -4162,7 +4204,7 @@
         <v>331</v>
       </c>
       <c r="C332" s="11" t="n">
-        <v>263</v>
+        <v>321</v>
       </c>
     </row>
     <row r="333" ht="11" customHeight="true" outlineLevel="3">
@@ -4170,7 +4212,7 @@
         <v>332</v>
       </c>
       <c r="C333" s="11" t="n">
-        <v>492</v>
+        <v>103</v>
       </c>
     </row>
     <row r="334" ht="11" customHeight="true" outlineLevel="3">
@@ -4178,7 +4220,7 @@
         <v>333</v>
       </c>
       <c r="C334" s="11" t="n">
-        <v>141</v>
+        <v>25</v>
       </c>
     </row>
     <row r="335" ht="11" customHeight="true" outlineLevel="3">
@@ -4186,7 +4228,7 @@
         <v>334</v>
       </c>
       <c r="C335" s="11" t="n">
-        <v>130</v>
+        <v>7</v>
       </c>
     </row>
     <row r="336" ht="11" customHeight="true" outlineLevel="3">
@@ -4194,23 +4236,23 @@
         <v>335</v>
       </c>
       <c r="C336" s="11" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="337" ht="22" customHeight="true" outlineLevel="3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="337" ht="11" customHeight="true" outlineLevel="3">
       <c r="B337" s="15" t="s">
         <v>336</v>
       </c>
       <c r="C337" s="11" t="n">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="338" ht="22" customHeight="true" outlineLevel="3">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="338" ht="11" customHeight="true" outlineLevel="3">
       <c r="B338" s="15" t="s">
         <v>337</v>
       </c>
       <c r="C338" s="11" t="n">
-        <v>79</v>
+        <v>274</v>
       </c>
     </row>
     <row r="339" ht="11" customHeight="true" outlineLevel="3">
@@ -4218,7 +4260,7 @@
         <v>338</v>
       </c>
       <c r="C339" s="11" t="n">
-        <v>11</v>
+        <v>322</v>
       </c>
     </row>
     <row r="340" ht="11" customHeight="true" outlineLevel="3">
@@ -4226,15 +4268,15 @@
         <v>339</v>
       </c>
       <c r="C340" s="11" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="341" ht="22" customHeight="true" outlineLevel="3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="341" ht="11" customHeight="true" outlineLevel="3">
       <c r="B341" s="15" t="s">
         <v>340</v>
       </c>
       <c r="C341" s="11" t="n">
-        <v>41</v>
+        <v>179</v>
       </c>
     </row>
     <row r="342" ht="11" customHeight="true" outlineLevel="3">
@@ -4242,15 +4284,15 @@
         <v>341</v>
       </c>
       <c r="C342" s="11" t="n">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="343" ht="22" customHeight="true" outlineLevel="3">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="343" ht="11" customHeight="true" outlineLevel="3">
       <c r="B343" s="15" t="s">
         <v>342</v>
       </c>
       <c r="C343" s="11" t="n">
-        <v>74</v>
+        <v>117</v>
       </c>
     </row>
     <row r="344" ht="11" customHeight="true" outlineLevel="3">
@@ -4258,23 +4300,23 @@
         <v>343</v>
       </c>
       <c r="C344" s="11" t="n">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="345" ht="22" customHeight="true" outlineLevel="3">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="345" ht="11" customHeight="true" outlineLevel="3">
       <c r="B345" s="15" t="s">
         <v>344</v>
       </c>
       <c r="C345" s="11" t="n">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="346" ht="11" customHeight="true" outlineLevel="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="346" ht="22" customHeight="true" outlineLevel="3">
       <c r="B346" s="15" t="s">
         <v>345</v>
       </c>
       <c r="C346" s="11" t="n">
-        <v>33</v>
+        <v>73</v>
       </c>
     </row>
     <row r="347" ht="22" customHeight="true" outlineLevel="3">
@@ -4282,15 +4324,15 @@
         <v>346</v>
       </c>
       <c r="C347" s="11" t="n">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="348" ht="11" customHeight="true" outlineLevel="3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="348" ht="22" customHeight="true" outlineLevel="3">
       <c r="B348" s="15" t="s">
         <v>347</v>
       </c>
       <c r="C348" s="11" t="n">
-        <v>47</v>
+        <v>21</v>
       </c>
     </row>
     <row r="349" ht="11" customHeight="true" outlineLevel="3">
@@ -4298,15 +4340,15 @@
         <v>348</v>
       </c>
       <c r="C349" s="11" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="350" ht="11" customHeight="true" outlineLevel="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="350" ht="22" customHeight="true" outlineLevel="3">
       <c r="B350" s="15" t="s">
         <v>349</v>
       </c>
       <c r="C350" s="11" t="n">
-        <v>56</v>
+        <v>46</v>
       </c>
     </row>
     <row r="351" ht="11" customHeight="true" outlineLevel="3">
@@ -4314,15 +4356,15 @@
         <v>350</v>
       </c>
       <c r="C351" s="11" t="n">
-        <v>859</v>
-      </c>
-    </row>
-    <row r="352" ht="11" customHeight="true" outlineLevel="3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="352" ht="22" customHeight="true" outlineLevel="3">
       <c r="B352" s="15" t="s">
         <v>351</v>
       </c>
-      <c r="C352" s="16" t="n">
-        <v>1757</v>
+      <c r="C352" s="11" t="n">
+        <v>72</v>
       </c>
     </row>
     <row r="353" ht="11" customHeight="true" outlineLevel="3">
@@ -4330,15 +4372,15 @@
         <v>352</v>
       </c>
       <c r="C353" s="11" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="354" ht="11" customHeight="true" outlineLevel="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="354" ht="22" customHeight="true" outlineLevel="3">
       <c r="B354" s="15" t="s">
         <v>353</v>
       </c>
       <c r="C354" s="11" t="n">
-        <v>493</v>
+        <v>29</v>
       </c>
     </row>
     <row r="355" ht="11" customHeight="true" outlineLevel="3">
@@ -4346,15 +4388,15 @@
         <v>354</v>
       </c>
       <c r="C355" s="11" t="n">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="356" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B356" s="14" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="356" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B356" s="15" t="s">
         <v>355</v>
       </c>
-      <c r="C356" s="17" t="n">
-        <v>89</v>
+      <c r="C356" s="11" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="357" ht="11" customHeight="true" outlineLevel="3">
@@ -4362,7 +4404,7 @@
         <v>356</v>
       </c>
       <c r="C357" s="11" t="n">
-        <v>75</v>
+        <v>225</v>
       </c>
     </row>
     <row r="358" ht="11" customHeight="true" outlineLevel="3">
@@ -4370,15 +4412,15 @@
         <v>357</v>
       </c>
       <c r="C358" s="11" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="359" ht="11" customHeight="true" outlineLevel="2">
-      <c r="B359" s="14" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="359" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B359" s="15" t="s">
         <v>358</v>
       </c>
-      <c r="C359" s="12" t="n">
-        <v>23118</v>
+      <c r="C359" s="16" t="n">
+        <v>1034</v>
       </c>
     </row>
     <row r="360" ht="11" customHeight="true" outlineLevel="3">
@@ -4386,7 +4428,7 @@
         <v>359</v>
       </c>
       <c r="C360" s="11" t="n">
-        <v>32</v>
+        <v>151</v>
       </c>
     </row>
     <row r="361" ht="11" customHeight="true" outlineLevel="3">
@@ -4394,7 +4436,7 @@
         <v>360</v>
       </c>
       <c r="C361" s="11" t="n">
-        <v>414</v>
+        <v>393</v>
       </c>
     </row>
     <row r="362" ht="11" customHeight="true" outlineLevel="3">
@@ -4402,47 +4444,47 @@
         <v>361</v>
       </c>
       <c r="C362" s="11" t="n">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="363" ht="22" customHeight="true" outlineLevel="3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="363" ht="11" customHeight="true" outlineLevel="3">
       <c r="B363" s="15" t="s">
         <v>362</v>
       </c>
       <c r="C363" s="11" t="n">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="364" ht="33" customHeight="true" outlineLevel="3">
-      <c r="B364" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="364" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B364" s="14" t="s">
         <v>363</v>
       </c>
-      <c r="C364" s="11" t="n">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="365" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C364" s="17" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="365" ht="11" customHeight="true" outlineLevel="3">
       <c r="B365" s="15" t="s">
         <v>364</v>
       </c>
       <c r="C365" s="11" t="n">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="366" ht="22" customHeight="true" outlineLevel="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="366" ht="11" customHeight="true" outlineLevel="3">
       <c r="B366" s="15" t="s">
         <v>365</v>
       </c>
       <c r="C366" s="11" t="n">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="367" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B367" s="15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="367" ht="11" customHeight="true" outlineLevel="2">
+      <c r="B367" s="14" t="s">
         <v>366</v>
       </c>
-      <c r="C367" s="11" t="n">
-        <v>606</v>
+      <c r="C367" s="12" t="n">
+        <v>22738</v>
       </c>
     </row>
     <row r="368" ht="11" customHeight="true" outlineLevel="3">
@@ -4450,15 +4492,15 @@
         <v>367</v>
       </c>
       <c r="C368" s="11" t="n">
-        <v>953</v>
-      </c>
-    </row>
-    <row r="369" ht="22" customHeight="true" outlineLevel="3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="369" ht="11" customHeight="true" outlineLevel="3">
       <c r="B369" s="15" t="s">
         <v>368</v>
       </c>
       <c r="C369" s="11" t="n">
-        <v>49</v>
+        <v>89</v>
       </c>
     </row>
     <row r="370" ht="22" customHeight="true" outlineLevel="3">
@@ -4466,47 +4508,47 @@
         <v>369</v>
       </c>
       <c r="C370" s="11" t="n">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="371" ht="11" customHeight="true" outlineLevel="3">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="371" ht="33" customHeight="true" outlineLevel="3">
       <c r="B371" s="15" t="s">
         <v>370</v>
       </c>
       <c r="C371" s="11" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="372" ht="11" customHeight="true" outlineLevel="3">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="372" ht="22" customHeight="true" outlineLevel="3">
       <c r="B372" s="15" t="s">
         <v>371</v>
       </c>
       <c r="C372" s="11" t="n">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="373" ht="11" customHeight="true" outlineLevel="3">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="373" ht="22" customHeight="true" outlineLevel="3">
       <c r="B373" s="15" t="s">
         <v>372</v>
       </c>
       <c r="C373" s="11" t="n">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="374" ht="22" customHeight="true" outlineLevel="3">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="374" ht="11" customHeight="true" outlineLevel="3">
       <c r="B374" s="15" t="s">
         <v>373</v>
       </c>
       <c r="C374" s="11" t="n">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="375" ht="22" customHeight="true" outlineLevel="3">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="375" ht="11" customHeight="true" outlineLevel="3">
       <c r="B375" s="15" t="s">
         <v>374</v>
       </c>
       <c r="C375" s="11" t="n">
-        <v>518</v>
+        <v>670</v>
       </c>
     </row>
     <row r="376" ht="22" customHeight="true" outlineLevel="3">
@@ -4514,31 +4556,31 @@
         <v>375</v>
       </c>
       <c r="C376" s="11" t="n">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="377" ht="22" customHeight="true" outlineLevel="3">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="377" ht="11" customHeight="true" outlineLevel="3">
       <c r="B377" s="15" t="s">
         <v>376</v>
       </c>
-      <c r="C377" s="16" t="n">
-        <v>1957</v>
-      </c>
-    </row>
-    <row r="378" ht="22" customHeight="true" outlineLevel="3">
+      <c r="C377" s="11" t="n">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="378" ht="11" customHeight="true" outlineLevel="3">
       <c r="B378" s="15" t="s">
         <v>377</v>
       </c>
       <c r="C378" s="11" t="n">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="379" ht="22" customHeight="true" outlineLevel="3">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="379" ht="11" customHeight="true" outlineLevel="3">
       <c r="B379" s="15" t="s">
         <v>378</v>
       </c>
-      <c r="C379" s="16" t="n">
-        <v>1572</v>
+      <c r="C379" s="11" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="380" ht="22" customHeight="true" outlineLevel="3">
@@ -4546,7 +4588,7 @@
         <v>379</v>
       </c>
       <c r="C380" s="11" t="n">
-        <v>113</v>
+        <v>159</v>
       </c>
     </row>
     <row r="381" ht="22" customHeight="true" outlineLevel="3">
@@ -4554,23 +4596,23 @@
         <v>380</v>
       </c>
       <c r="C381" s="11" t="n">
-        <v>18</v>
+        <v>167</v>
       </c>
     </row>
     <row r="382" ht="22" customHeight="true" outlineLevel="3">
       <c r="B382" s="15" t="s">
         <v>381</v>
       </c>
-      <c r="C382" s="16" t="n">
-        <v>1534</v>
+      <c r="C382" s="11" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="383" ht="22" customHeight="true" outlineLevel="3">
       <c r="B383" s="15" t="s">
         <v>382</v>
       </c>
-      <c r="C383" s="11" t="n">
-        <v>183</v>
+      <c r="C383" s="16" t="n">
+        <v>1174</v>
       </c>
     </row>
     <row r="384" ht="22" customHeight="true" outlineLevel="3">
@@ -4578,23 +4620,23 @@
         <v>383</v>
       </c>
       <c r="C384" s="11" t="n">
-        <v>102</v>
+        <v>512</v>
       </c>
     </row>
     <row r="385" ht="22" customHeight="true" outlineLevel="3">
       <c r="B385" s="15" t="s">
         <v>384</v>
       </c>
-      <c r="C385" s="11" t="n">
-        <v>39</v>
+      <c r="C385" s="16" t="n">
+        <v>1137</v>
       </c>
     </row>
     <row r="386" ht="22" customHeight="true" outlineLevel="3">
       <c r="B386" s="15" t="s">
         <v>385</v>
       </c>
-      <c r="C386" s="16" t="n">
-        <v>1450</v>
+      <c r="C386" s="11" t="n">
+        <v>90</v>
       </c>
     </row>
     <row r="387" ht="22" customHeight="true" outlineLevel="3">
@@ -4602,15 +4644,15 @@
         <v>386</v>
       </c>
       <c r="C387" s="11" t="n">
-        <v>81</v>
+        <v>18</v>
       </c>
     </row>
     <row r="388" ht="22" customHeight="true" outlineLevel="3">
       <c r="B388" s="15" t="s">
         <v>387</v>
       </c>
-      <c r="C388" s="11" t="n">
-        <v>7</v>
+      <c r="C388" s="16" t="n">
+        <v>1171</v>
       </c>
     </row>
     <row r="389" ht="22" customHeight="true" outlineLevel="3">
@@ -4618,7 +4660,7 @@
         <v>388</v>
       </c>
       <c r="C389" s="11" t="n">
-        <v>44</v>
+        <v>342</v>
       </c>
     </row>
     <row r="390" ht="22" customHeight="true" outlineLevel="3">
@@ -4626,7 +4668,7 @@
         <v>389</v>
       </c>
       <c r="C390" s="11" t="n">
-        <v>152</v>
+        <v>102</v>
       </c>
     </row>
     <row r="391" ht="22" customHeight="true" outlineLevel="3">
@@ -4634,7 +4676,7 @@
         <v>390</v>
       </c>
       <c r="C391" s="11" t="n">
-        <v>66</v>
+        <v>39</v>
       </c>
     </row>
     <row r="392" ht="22" customHeight="true" outlineLevel="3">
@@ -4642,7 +4684,7 @@
         <v>391</v>
       </c>
       <c r="C392" s="16" t="n">
-        <v>2681</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="393" ht="22" customHeight="true" outlineLevel="3">
@@ -4650,23 +4692,23 @@
         <v>392</v>
       </c>
       <c r="C393" s="11" t="n">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="394" ht="11" customHeight="true" outlineLevel="3">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="394" ht="22" customHeight="true" outlineLevel="3">
       <c r="B394" s="15" t="s">
         <v>393</v>
       </c>
       <c r="C394" s="11" t="n">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="395" ht="11" customHeight="true" outlineLevel="3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="395" ht="22" customHeight="true" outlineLevel="3">
       <c r="B395" s="15" t="s">
         <v>394</v>
       </c>
       <c r="C395" s="11" t="n">
-        <v>140</v>
+        <v>44</v>
       </c>
     </row>
     <row r="396" ht="22" customHeight="true" outlineLevel="3">
@@ -4674,7 +4716,7 @@
         <v>395</v>
       </c>
       <c r="C396" s="11" t="n">
-        <v>52</v>
+        <v>123</v>
       </c>
     </row>
     <row r="397" ht="22" customHeight="true" outlineLevel="3">
@@ -4682,15 +4724,15 @@
         <v>396</v>
       </c>
       <c r="C397" s="11" t="n">
-        <v>13</v>
+        <v>66</v>
       </c>
     </row>
     <row r="398" ht="22" customHeight="true" outlineLevel="3">
       <c r="B398" s="15" t="s">
         <v>397</v>
       </c>
-      <c r="C398" s="11" t="n">
-        <v>10</v>
+      <c r="C398" s="16" t="n">
+        <v>1154</v>
       </c>
     </row>
     <row r="399" ht="22" customHeight="true" outlineLevel="3">
@@ -4698,23 +4740,23 @@
         <v>398</v>
       </c>
       <c r="C399" s="11" t="n">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="400" ht="22" customHeight="true" outlineLevel="3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="400" ht="11" customHeight="true" outlineLevel="3">
       <c r="B400" s="15" t="s">
         <v>399</v>
       </c>
       <c r="C400" s="11" t="n">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="401" ht="22" customHeight="true" outlineLevel="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="401" ht="11" customHeight="true" outlineLevel="3">
       <c r="B401" s="15" t="s">
         <v>400</v>
       </c>
       <c r="C401" s="11" t="n">
-        <v>201</v>
+        <v>191</v>
       </c>
     </row>
     <row r="402" ht="22" customHeight="true" outlineLevel="3">
@@ -4722,55 +4764,55 @@
         <v>401</v>
       </c>
       <c r="C402" s="11" t="n">
-        <v>870</v>
-      </c>
-    </row>
-    <row r="403" ht="11" customHeight="true" outlineLevel="3">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="403" ht="22" customHeight="true" outlineLevel="3">
       <c r="B403" s="15" t="s">
         <v>402</v>
       </c>
       <c r="C403" s="11" t="n">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="404" ht="11" customHeight="true" outlineLevel="3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="404" ht="22" customHeight="true" outlineLevel="3">
       <c r="B404" s="15" t="s">
         <v>403</v>
       </c>
       <c r="C404" s="11" t="n">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="405" ht="11" customHeight="true" outlineLevel="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="405" ht="22" customHeight="true" outlineLevel="3">
       <c r="B405" s="15" t="s">
         <v>404</v>
       </c>
       <c r="C405" s="11" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="406" ht="11" customHeight="true" outlineLevel="3">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="406" ht="22" customHeight="true" outlineLevel="3">
       <c r="B406" s="15" t="s">
         <v>405</v>
       </c>
       <c r="C406" s="11" t="n">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="407" ht="11" customHeight="true" outlineLevel="3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="407" ht="22" customHeight="true" outlineLevel="3">
       <c r="B407" s="15" t="s">
         <v>406</v>
       </c>
       <c r="C407" s="11" t="n">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="408" ht="11" customHeight="true" outlineLevel="3">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="408" ht="22" customHeight="true" outlineLevel="3">
       <c r="B408" s="15" t="s">
         <v>407</v>
       </c>
       <c r="C408" s="11" t="n">
-        <v>601</v>
+        <v>609</v>
       </c>
     </row>
     <row r="409" ht="11" customHeight="true" outlineLevel="3">
@@ -4778,15 +4820,15 @@
         <v>408</v>
       </c>
       <c r="C409" s="11" t="n">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="410" ht="11" customHeight="true" outlineLevel="3">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="410" ht="22" customHeight="true" outlineLevel="3">
       <c r="B410" s="15" t="s">
         <v>409</v>
       </c>
-      <c r="C410" s="11" t="n">
-        <v>184</v>
+      <c r="C410" s="16" t="n">
+        <v>1045</v>
       </c>
     </row>
     <row r="411" ht="11" customHeight="true" outlineLevel="3">
@@ -4794,15 +4836,15 @@
         <v>410</v>
       </c>
       <c r="C411" s="11" t="n">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="412" ht="11" customHeight="true" outlineLevel="3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="412" ht="22" customHeight="true" outlineLevel="3">
       <c r="B412" s="15" t="s">
         <v>411</v>
       </c>
       <c r="C412" s="11" t="n">
-        <v>299</v>
+        <v>748</v>
       </c>
     </row>
     <row r="413" ht="11" customHeight="true" outlineLevel="3">
@@ -4810,15 +4852,15 @@
         <v>412</v>
       </c>
       <c r="C413" s="11" t="n">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="414" ht="11" customHeight="true" outlineLevel="3">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="414" ht="22" customHeight="true" outlineLevel="3">
       <c r="B414" s="15" t="s">
         <v>413</v>
       </c>
       <c r="C414" s="11" t="n">
-        <v>211</v>
+        <v>874</v>
       </c>
     </row>
     <row r="415" ht="11" customHeight="true" outlineLevel="3">
@@ -4826,47 +4868,159 @@
         <v>414</v>
       </c>
       <c r="C415" s="11" t="n">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="416" ht="11" customHeight="true" outlineLevel="3">
-      <c r="B416" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="416" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B416" s="15" t="s">
         <v>415</v>
       </c>
-      <c r="C416" s="12" t="n">
-        <v>1727</v>
-      </c>
-    </row>
-    <row r="417" ht="11" customHeight="true" outlineLevel="4">
-      <c r="B417" s="19" t="s">
+      <c r="C416" s="11" t="n">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="417" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B417" s="15" t="s">
         <v>416</v>
       </c>
       <c r="C417" s="11" t="n">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="418" ht="11" customHeight="true" outlineLevel="4">
-      <c r="B418" s="19" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="418" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B418" s="15" t="s">
         <v>417</v>
       </c>
       <c r="C418" s="11" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="419" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B419" s="15" t="s">
+        <v>418</v>
+      </c>
+      <c r="C419" s="11" t="n">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="420" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B420" s="15" t="s">
+        <v>419</v>
+      </c>
+      <c r="C420" s="11" t="n">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="421" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B421" s="15" t="s">
+        <v>420</v>
+      </c>
+      <c r="C421" s="11" t="n">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="422" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B422" s="15" t="s">
+        <v>421</v>
+      </c>
+      <c r="C422" s="11" t="n">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="423" ht="22" customHeight="true" outlineLevel="3">
+      <c r="B423" s="15" t="s">
+        <v>422</v>
+      </c>
+      <c r="C423" s="16" t="n">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="424" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B424" s="15" t="s">
+        <v>423</v>
+      </c>
+      <c r="C424" s="11" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="425" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B425" s="15" t="s">
+        <v>424</v>
+      </c>
+      <c r="C425" s="11" t="n">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="426" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B426" s="15" t="s">
+        <v>425</v>
+      </c>
+      <c r="C426" s="11" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="427" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B427" s="15" t="s">
+        <v>426</v>
+      </c>
+      <c r="C427" s="11" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="428" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B428" s="15" t="s">
+        <v>427</v>
+      </c>
+      <c r="C428" s="11" t="n">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="429" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B429" s="15" t="s">
+        <v>428</v>
+      </c>
+      <c r="C429" s="11" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="430" ht="11" customHeight="true" outlineLevel="3">
+      <c r="B430" s="18" t="s">
+        <v>429</v>
+      </c>
+      <c r="C430" s="17" t="n">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="431" ht="11" customHeight="true" outlineLevel="4">
+      <c r="B431" s="19" t="s">
+        <v>430</v>
+      </c>
+      <c r="C431" s="11" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="419" ht="11" customHeight="true" outlineLevel="4">
-      <c r="B419" s="19" t="s">
-        <v>418</v>
-      </c>
-      <c r="C419" s="11" t="n">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="420" ht="11" customHeight="true" outlineLevel="4">
-      <c r="B420" s="19" t="s">
-        <v>419</v>
-      </c>
-      <c r="C420" s="11" t="n">
-        <v>200</v>
+    <row r="432" ht="11" customHeight="true" outlineLevel="4">
+      <c r="B432" s="19" t="s">
+        <v>431</v>
+      </c>
+      <c r="C432" s="11" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="433" ht="11" customHeight="true" outlineLevel="4">
+      <c r="B433" s="19" t="s">
+        <v>432</v>
+      </c>
+      <c r="C433" s="11" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="434" ht="11" customHeight="true" outlineLevel="4">
+      <c r="B434" s="19" t="s">
+        <v>433</v>
+      </c>
+      <c r="C434" s="11" t="n">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>